<commit_message>
docs(commercial): finaliser préparation campagne pilote ELSATIA
</commit_message>
<xml_diff>
--- a/docs/commercial/C5D_MODELE_SUIVI_CAMPAGNE_PILOTE_ELSATIA.xlsx
+++ b/docs/commercial/C5D_MODELE_SUIVI_CAMPAGNE_PILOTE_ELSATIA.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1ca049f04d1044df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROSPECTS" sheetId="2" r:id="R040b464e7db54113"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIONS" sheetId="3" r:id="R09936f55d23a45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPPOSITIONS" sheetId="4" r:id="Rd6a70ec5071a4776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLEAU_DE_BORD" sheetId="5" r:id="Rc019ffc8a17449a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTES" sheetId="6" r:id="Ra2db092c6a374733"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R48b68ccb981f4cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROSPECTS" sheetId="2" r:id="R5f2d04a6b2af471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIONS" sheetId="3" r:id="Rcb82c40fed024b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPPOSITIONS" sheetId="4" r:id="R367c1234ab8d4dad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLEAU_DE_BORD" sheetId="5" r:id="R88989e0a06794734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTES" sheetId="6" r:id="R3b91254b6d9d41d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +24,7 @@
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -87,8 +87,14 @@
       <x:color rgb="FF15233B"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -150,8 +156,13 @@
         <x:fgColor rgb="FFFFF8EC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3478F6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -196,11 +207,25 @@
         <x:color rgb="FF10213F"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD6E2F4"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD6E2F4"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD6E2F4"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6E2F4"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -390,6 +415,15 @@
     <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -401,7 +435,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE3E3"/>
         </x:patternFill>
       </x:fill>
@@ -412,7 +446,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE3E3"/>
         </x:patternFill>
       </x:fill>
@@ -423,7 +457,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDFF3E5"/>
         </x:patternFill>
       </x:fill>
@@ -434,7 +468,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE3E3"/>
         </x:patternFill>
       </x:fill>
@@ -797,7 +831,7 @@
         <x:v>1. Avant toute collecte</x:v>
       </x:c>
       <x:c r="B7" s="20" t="str">
-        <x:v>Compléter la checklist GO / NO-GO C5-D. Une case manquante interdit la collecte.</x:v>
+        <x:v>Responsable : Julien GREGUREC. Destination : ELSATIA / Commercial / Prospection / Campagne pilote, accès restreint.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -821,7 +855,7 @@
         <x:v>4. Qualifier</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>Conserver seulement les P1/P2 sans motif d’exclusion pour les lots pilotes.</x:v>
+        <x:v>P1/P2 seulement dans les lots. P3 (45–59) signifie à enrichir avant tout contact.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -829,7 +863,7 @@
         <x:v>5. Contrôler l’opposition</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>Rechercher l’identifiant minimal dans OPPOSITIONS avant ajout, gel de lot et action.</x:v>
+        <x:v>Rechercher l’identifiant minimal dans OPPOSITIONS avant ajout, gel de lot et action ; statut NE PLUS CONTACTER.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -837,7 +871,7 @@
         <x:v>6. Contacter</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Envoi manuel et personnalisé depuis la boîte professionnelle validée. Aucun automatisme.</x:v>
+        <x:v>Envoi manuel, unitaire et personnalisé via Google Workspace depuis contact@elsatia.fr. Aucun automatisme.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -869,7 +903,7 @@
         <x:v>10. Revue</x:v>
       </x:c>
       <x:c r="B16" s="21" t="str">
-        <x:v>Analyser chaque lot de 10 avant d’autoriser le suivant.</x:v>
+        <x:v>Cadence J0, J3, J5, J8, J13 ; décaler au prochain jour ouvré si nécessaire et revoir chaque lot de 10.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -877,7 +911,7 @@
         <x:v>11. Conservation</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>Appliquer uniquement la politique validée avant lancement ; supprimer ou anonymiser à l’échéance.</x:v>
+        <x:v>Prospects : 3 ans maximum depuis la collecte ou le dernier contact pertinent, avec suppression anticipée si inutile. Opposition : 3 ans minimum.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -885,7 +919,7 @@
         <x:v>12. Interdit</x:v>
       </x:c>
       <x:c r="B18" s="21" t="str">
-        <x:v>Aucune donnée personnelle inutile, privée, sensible, Production ou secrète.</x:v>
+        <x:v>Données professionnelles minimales uniquement ; aucune donnée privée, sensible, Production ou secrète.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -957,7 +991,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B28" s="21" t="str">
-        <x:v>C5-D · modèle vide · 2026-08-15</x:v>
+        <x:v>C5-D · modèle vide finalisé · 2026-08-15</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1439,7 +1473,7 @@
         <x:f>IF(AF6&gt;=7,SUM(V6:AE6),"")</x:f>
       </x:c>
       <x:c r="AH6" s="32" t="str">
-        <x:f>IF(AF6&lt;7,"À rechercher",IF(AG6&gt;=75,"P1",IF(AG6&gt;=60,"P2",IF(AG6&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF6&lt;7,"À rechercher",IF(AG6&gt;=75,"P1",IF(AG6&gt;=60,"P2",IF(AG6&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI6" s="30"/>
@@ -1510,7 +1544,7 @@
         <x:f>IF(AF7&gt;=7,SUM(V7:AE7),"")</x:f>
       </x:c>
       <x:c r="AH7" s="33" t="str">
-        <x:f>IF(AF7&lt;7,"À rechercher",IF(AG7&gt;=75,"P2",IF(AG7&gt;=60,"P3",IF(AG7&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF7&lt;7,"À rechercher",IF(AG7&gt;=75,"P1",IF(AG7&gt;=60,"P2",IF(AG7&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI7" s="31"/>
@@ -1581,7 +1615,7 @@
         <x:f>IF(AF8&gt;=7,SUM(V8:AE8),"")</x:f>
       </x:c>
       <x:c r="AH8" s="33" t="str">
-        <x:f>IF(AF8&lt;7,"À rechercher",IF(AG8&gt;=75,"P3",IF(AG8&gt;=60,"P4",IF(AG8&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF8&lt;7,"À rechercher",IF(AG8&gt;=75,"P1",IF(AG8&gt;=60,"P2",IF(AG8&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI8" s="31"/>
@@ -1652,7 +1686,7 @@
         <x:f>IF(AF9&gt;=7,SUM(V9:AE9),"")</x:f>
       </x:c>
       <x:c r="AH9" s="33" t="str">
-        <x:f>IF(AF9&lt;7,"À rechercher",IF(AG9&gt;=75,"P4",IF(AG9&gt;=60,"P5",IF(AG9&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF9&lt;7,"À rechercher",IF(AG9&gt;=75,"P1",IF(AG9&gt;=60,"P2",IF(AG9&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI9" s="31"/>
@@ -1723,7 +1757,7 @@
         <x:f>IF(AF10&gt;=7,SUM(V10:AE10),"")</x:f>
       </x:c>
       <x:c r="AH10" s="33" t="str">
-        <x:f>IF(AF10&lt;7,"À rechercher",IF(AG10&gt;=75,"P5",IF(AG10&gt;=60,"P6",IF(AG10&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF10&lt;7,"À rechercher",IF(AG10&gt;=75,"P1",IF(AG10&gt;=60,"P2",IF(AG10&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI10" s="31"/>
@@ -1794,7 +1828,7 @@
         <x:f>IF(AF11&gt;=7,SUM(V11:AE11),"")</x:f>
       </x:c>
       <x:c r="AH11" s="33" t="str">
-        <x:f>IF(AF11&lt;7,"À rechercher",IF(AG11&gt;=75,"P6",IF(AG11&gt;=60,"P7",IF(AG11&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF11&lt;7,"À rechercher",IF(AG11&gt;=75,"P1",IF(AG11&gt;=60,"P2",IF(AG11&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI11" s="31"/>
@@ -1865,7 +1899,7 @@
         <x:f>IF(AF12&gt;=7,SUM(V12:AE12),"")</x:f>
       </x:c>
       <x:c r="AH12" s="33" t="str">
-        <x:f>IF(AF12&lt;7,"À rechercher",IF(AG12&gt;=75,"P7",IF(AG12&gt;=60,"P8",IF(AG12&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF12&lt;7,"À rechercher",IF(AG12&gt;=75,"P1",IF(AG12&gt;=60,"P2",IF(AG12&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI12" s="31"/>
@@ -1936,7 +1970,7 @@
         <x:f>IF(AF13&gt;=7,SUM(V13:AE13),"")</x:f>
       </x:c>
       <x:c r="AH13" s="33" t="str">
-        <x:f>IF(AF13&lt;7,"À rechercher",IF(AG13&gt;=75,"P8",IF(AG13&gt;=60,"P9",IF(AG13&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF13&lt;7,"À rechercher",IF(AG13&gt;=75,"P1",IF(AG13&gt;=60,"P2",IF(AG13&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI13" s="31"/>
@@ -2007,7 +2041,7 @@
         <x:f>IF(AF14&gt;=7,SUM(V14:AE14),"")</x:f>
       </x:c>
       <x:c r="AH14" s="33" t="str">
-        <x:f>IF(AF14&lt;7,"À rechercher",IF(AG14&gt;=75,"P9",IF(AG14&gt;=60,"P10",IF(AG14&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF14&lt;7,"À rechercher",IF(AG14&gt;=75,"P1",IF(AG14&gt;=60,"P2",IF(AG14&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI14" s="31"/>
@@ -2078,7 +2112,7 @@
         <x:f>IF(AF15&gt;=7,SUM(V15:AE15),"")</x:f>
       </x:c>
       <x:c r="AH15" s="33" t="str">
-        <x:f>IF(AF15&lt;7,"À rechercher",IF(AG15&gt;=75,"P10",IF(AG15&gt;=60,"P11",IF(AG15&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF15&lt;7,"À rechercher",IF(AG15&gt;=75,"P1",IF(AG15&gt;=60,"P2",IF(AG15&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI15" s="31"/>
@@ -2149,7 +2183,7 @@
         <x:f>IF(AF16&gt;=7,SUM(V16:AE16),"")</x:f>
       </x:c>
       <x:c r="AH16" s="33" t="str">
-        <x:f>IF(AF16&lt;7,"À rechercher",IF(AG16&gt;=75,"P11",IF(AG16&gt;=60,"P12",IF(AG16&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF16&lt;7,"À rechercher",IF(AG16&gt;=75,"P1",IF(AG16&gt;=60,"P2",IF(AG16&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI16" s="31"/>
@@ -2220,7 +2254,7 @@
         <x:f>IF(AF17&gt;=7,SUM(V17:AE17),"")</x:f>
       </x:c>
       <x:c r="AH17" s="33" t="str">
-        <x:f>IF(AF17&lt;7,"À rechercher",IF(AG17&gt;=75,"P12",IF(AG17&gt;=60,"P13",IF(AG17&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF17&lt;7,"À rechercher",IF(AG17&gt;=75,"P1",IF(AG17&gt;=60,"P2",IF(AG17&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI17" s="31"/>
@@ -2291,7 +2325,7 @@
         <x:f>IF(AF18&gt;=7,SUM(V18:AE18),"")</x:f>
       </x:c>
       <x:c r="AH18" s="33" t="str">
-        <x:f>IF(AF18&lt;7,"À rechercher",IF(AG18&gt;=75,"P13",IF(AG18&gt;=60,"P14",IF(AG18&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF18&lt;7,"À rechercher",IF(AG18&gt;=75,"P1",IF(AG18&gt;=60,"P2",IF(AG18&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI18" s="31"/>
@@ -2362,7 +2396,7 @@
         <x:f>IF(AF19&gt;=7,SUM(V19:AE19),"")</x:f>
       </x:c>
       <x:c r="AH19" s="33" t="str">
-        <x:f>IF(AF19&lt;7,"À rechercher",IF(AG19&gt;=75,"P14",IF(AG19&gt;=60,"P15",IF(AG19&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF19&lt;7,"À rechercher",IF(AG19&gt;=75,"P1",IF(AG19&gt;=60,"P2",IF(AG19&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI19" s="31"/>
@@ -2433,7 +2467,7 @@
         <x:f>IF(AF20&gt;=7,SUM(V20:AE20),"")</x:f>
       </x:c>
       <x:c r="AH20" s="33" t="str">
-        <x:f>IF(AF20&lt;7,"À rechercher",IF(AG20&gt;=75,"P15",IF(AG20&gt;=60,"P16",IF(AG20&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF20&lt;7,"À rechercher",IF(AG20&gt;=75,"P1",IF(AG20&gt;=60,"P2",IF(AG20&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI20" s="31"/>
@@ -2504,7 +2538,7 @@
         <x:f>IF(AF21&gt;=7,SUM(V21:AE21),"")</x:f>
       </x:c>
       <x:c r="AH21" s="33" t="str">
-        <x:f>IF(AF21&lt;7,"À rechercher",IF(AG21&gt;=75,"P16",IF(AG21&gt;=60,"P17",IF(AG21&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF21&lt;7,"À rechercher",IF(AG21&gt;=75,"P1",IF(AG21&gt;=60,"P2",IF(AG21&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI21" s="31"/>
@@ -2575,7 +2609,7 @@
         <x:f>IF(AF22&gt;=7,SUM(V22:AE22),"")</x:f>
       </x:c>
       <x:c r="AH22" s="33" t="str">
-        <x:f>IF(AF22&lt;7,"À rechercher",IF(AG22&gt;=75,"P17",IF(AG22&gt;=60,"P18",IF(AG22&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF22&lt;7,"À rechercher",IF(AG22&gt;=75,"P1",IF(AG22&gt;=60,"P2",IF(AG22&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI22" s="31"/>
@@ -2646,7 +2680,7 @@
         <x:f>IF(AF23&gt;=7,SUM(V23:AE23),"")</x:f>
       </x:c>
       <x:c r="AH23" s="33" t="str">
-        <x:f>IF(AF23&lt;7,"À rechercher",IF(AG23&gt;=75,"P18",IF(AG23&gt;=60,"P19",IF(AG23&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF23&lt;7,"À rechercher",IF(AG23&gt;=75,"P1",IF(AG23&gt;=60,"P2",IF(AG23&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI23" s="31"/>
@@ -2717,7 +2751,7 @@
         <x:f>IF(AF24&gt;=7,SUM(V24:AE24),"")</x:f>
       </x:c>
       <x:c r="AH24" s="33" t="str">
-        <x:f>IF(AF24&lt;7,"À rechercher",IF(AG24&gt;=75,"P19",IF(AG24&gt;=60,"P20",IF(AG24&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF24&lt;7,"À rechercher",IF(AG24&gt;=75,"P1",IF(AG24&gt;=60,"P2",IF(AG24&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI24" s="31"/>
@@ -2788,7 +2822,7 @@
         <x:f>IF(AF25&gt;=7,SUM(V25:AE25),"")</x:f>
       </x:c>
       <x:c r="AH25" s="33" t="str">
-        <x:f>IF(AF25&lt;7,"À rechercher",IF(AG25&gt;=75,"P20",IF(AG25&gt;=60,"P21",IF(AG25&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF25&lt;7,"À rechercher",IF(AG25&gt;=75,"P1",IF(AG25&gt;=60,"P2",IF(AG25&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI25" s="31"/>
@@ -2859,7 +2893,7 @@
         <x:f>IF(AF26&gt;=7,SUM(V26:AE26),"")</x:f>
       </x:c>
       <x:c r="AH26" s="33" t="str">
-        <x:f>IF(AF26&lt;7,"À rechercher",IF(AG26&gt;=75,"P21",IF(AG26&gt;=60,"P22",IF(AG26&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF26&lt;7,"À rechercher",IF(AG26&gt;=75,"P1",IF(AG26&gt;=60,"P2",IF(AG26&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI26" s="31"/>
@@ -2930,7 +2964,7 @@
         <x:f>IF(AF27&gt;=7,SUM(V27:AE27),"")</x:f>
       </x:c>
       <x:c r="AH27" s="33" t="str">
-        <x:f>IF(AF27&lt;7,"À rechercher",IF(AG27&gt;=75,"P22",IF(AG27&gt;=60,"P23",IF(AG27&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF27&lt;7,"À rechercher",IF(AG27&gt;=75,"P1",IF(AG27&gt;=60,"P2",IF(AG27&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI27" s="31"/>
@@ -3001,7 +3035,7 @@
         <x:f>IF(AF28&gt;=7,SUM(V28:AE28),"")</x:f>
       </x:c>
       <x:c r="AH28" s="33" t="str">
-        <x:f>IF(AF28&lt;7,"À rechercher",IF(AG28&gt;=75,"P23",IF(AG28&gt;=60,"P24",IF(AG28&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF28&lt;7,"À rechercher",IF(AG28&gt;=75,"P1",IF(AG28&gt;=60,"P2",IF(AG28&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI28" s="31"/>
@@ -3072,7 +3106,7 @@
         <x:f>IF(AF29&gt;=7,SUM(V29:AE29),"")</x:f>
       </x:c>
       <x:c r="AH29" s="33" t="str">
-        <x:f>IF(AF29&lt;7,"À rechercher",IF(AG29&gt;=75,"P24",IF(AG29&gt;=60,"P25",IF(AG29&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF29&lt;7,"À rechercher",IF(AG29&gt;=75,"P1",IF(AG29&gt;=60,"P2",IF(AG29&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI29" s="31"/>
@@ -3143,7 +3177,7 @@
         <x:f>IF(AF30&gt;=7,SUM(V30:AE30),"")</x:f>
       </x:c>
       <x:c r="AH30" s="33" t="str">
-        <x:f>IF(AF30&lt;7,"À rechercher",IF(AG30&gt;=75,"P25",IF(AG30&gt;=60,"P26",IF(AG30&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF30&lt;7,"À rechercher",IF(AG30&gt;=75,"P1",IF(AG30&gt;=60,"P2",IF(AG30&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI30" s="31"/>
@@ -3214,7 +3248,7 @@
         <x:f>IF(AF31&gt;=7,SUM(V31:AE31),"")</x:f>
       </x:c>
       <x:c r="AH31" s="33" t="str">
-        <x:f>IF(AF31&lt;7,"À rechercher",IF(AG31&gt;=75,"P26",IF(AG31&gt;=60,"P27",IF(AG31&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF31&lt;7,"À rechercher",IF(AG31&gt;=75,"P1",IF(AG31&gt;=60,"P2",IF(AG31&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI31" s="31"/>
@@ -3285,7 +3319,7 @@
         <x:f>IF(AF32&gt;=7,SUM(V32:AE32),"")</x:f>
       </x:c>
       <x:c r="AH32" s="33" t="str">
-        <x:f>IF(AF32&lt;7,"À rechercher",IF(AG32&gt;=75,"P27",IF(AG32&gt;=60,"P28",IF(AG32&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF32&lt;7,"À rechercher",IF(AG32&gt;=75,"P1",IF(AG32&gt;=60,"P2",IF(AG32&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI32" s="31"/>
@@ -3356,7 +3390,7 @@
         <x:f>IF(AF33&gt;=7,SUM(V33:AE33),"")</x:f>
       </x:c>
       <x:c r="AH33" s="33" t="str">
-        <x:f>IF(AF33&lt;7,"À rechercher",IF(AG33&gt;=75,"P28",IF(AG33&gt;=60,"P29",IF(AG33&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF33&lt;7,"À rechercher",IF(AG33&gt;=75,"P1",IF(AG33&gt;=60,"P2",IF(AG33&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI33" s="31"/>
@@ -3427,7 +3461,7 @@
         <x:f>IF(AF34&gt;=7,SUM(V34:AE34),"")</x:f>
       </x:c>
       <x:c r="AH34" s="33" t="str">
-        <x:f>IF(AF34&lt;7,"À rechercher",IF(AG34&gt;=75,"P29",IF(AG34&gt;=60,"P30",IF(AG34&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF34&lt;7,"À rechercher",IF(AG34&gt;=75,"P1",IF(AG34&gt;=60,"P2",IF(AG34&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI34" s="31"/>
@@ -3498,7 +3532,7 @@
         <x:f>IF(AF35&gt;=7,SUM(V35:AE35),"")</x:f>
       </x:c>
       <x:c r="AH35" s="33" t="str">
-        <x:f>IF(AF35&lt;7,"À rechercher",IF(AG35&gt;=75,"P30",IF(AG35&gt;=60,"P31",IF(AG35&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF35&lt;7,"À rechercher",IF(AG35&gt;=75,"P1",IF(AG35&gt;=60,"P2",IF(AG35&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI35" s="31"/>
@@ -3569,7 +3603,7 @@
         <x:f>IF(AF36&gt;=7,SUM(V36:AE36),"")</x:f>
       </x:c>
       <x:c r="AH36" s="33" t="str">
-        <x:f>IF(AF36&lt;7,"À rechercher",IF(AG36&gt;=75,"P31",IF(AG36&gt;=60,"P32",IF(AG36&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF36&lt;7,"À rechercher",IF(AG36&gt;=75,"P1",IF(AG36&gt;=60,"P2",IF(AG36&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI36" s="31"/>
@@ -3640,7 +3674,7 @@
         <x:f>IF(AF37&gt;=7,SUM(V37:AE37),"")</x:f>
       </x:c>
       <x:c r="AH37" s="33" t="str">
-        <x:f>IF(AF37&lt;7,"À rechercher",IF(AG37&gt;=75,"P32",IF(AG37&gt;=60,"P33",IF(AG37&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF37&lt;7,"À rechercher",IF(AG37&gt;=75,"P1",IF(AG37&gt;=60,"P2",IF(AG37&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI37" s="31"/>
@@ -3711,7 +3745,7 @@
         <x:f>IF(AF38&gt;=7,SUM(V38:AE38),"")</x:f>
       </x:c>
       <x:c r="AH38" s="33" t="str">
-        <x:f>IF(AF38&lt;7,"À rechercher",IF(AG38&gt;=75,"P33",IF(AG38&gt;=60,"P34",IF(AG38&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF38&lt;7,"À rechercher",IF(AG38&gt;=75,"P1",IF(AG38&gt;=60,"P2",IF(AG38&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI38" s="31"/>
@@ -3782,7 +3816,7 @@
         <x:f>IF(AF39&gt;=7,SUM(V39:AE39),"")</x:f>
       </x:c>
       <x:c r="AH39" s="33" t="str">
-        <x:f>IF(AF39&lt;7,"À rechercher",IF(AG39&gt;=75,"P34",IF(AG39&gt;=60,"P35",IF(AG39&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF39&lt;7,"À rechercher",IF(AG39&gt;=75,"P1",IF(AG39&gt;=60,"P2",IF(AG39&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI39" s="31"/>
@@ -3853,7 +3887,7 @@
         <x:f>IF(AF40&gt;=7,SUM(V40:AE40),"")</x:f>
       </x:c>
       <x:c r="AH40" s="33" t="str">
-        <x:f>IF(AF40&lt;7,"À rechercher",IF(AG40&gt;=75,"P35",IF(AG40&gt;=60,"P36",IF(AG40&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF40&lt;7,"À rechercher",IF(AG40&gt;=75,"P1",IF(AG40&gt;=60,"P2",IF(AG40&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI40" s="31"/>
@@ -3924,7 +3958,7 @@
         <x:f>IF(AF41&gt;=7,SUM(V41:AE41),"")</x:f>
       </x:c>
       <x:c r="AH41" s="33" t="str">
-        <x:f>IF(AF41&lt;7,"À rechercher",IF(AG41&gt;=75,"P36",IF(AG41&gt;=60,"P37",IF(AG41&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF41&lt;7,"À rechercher",IF(AG41&gt;=75,"P1",IF(AG41&gt;=60,"P2",IF(AG41&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI41" s="31"/>
@@ -3995,7 +4029,7 @@
         <x:f>IF(AF42&gt;=7,SUM(V42:AE42),"")</x:f>
       </x:c>
       <x:c r="AH42" s="33" t="str">
-        <x:f>IF(AF42&lt;7,"À rechercher",IF(AG42&gt;=75,"P37",IF(AG42&gt;=60,"P38",IF(AG42&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF42&lt;7,"À rechercher",IF(AG42&gt;=75,"P1",IF(AG42&gt;=60,"P2",IF(AG42&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI42" s="31"/>
@@ -4066,7 +4100,7 @@
         <x:f>IF(AF43&gt;=7,SUM(V43:AE43),"")</x:f>
       </x:c>
       <x:c r="AH43" s="33" t="str">
-        <x:f>IF(AF43&lt;7,"À rechercher",IF(AG43&gt;=75,"P38",IF(AG43&gt;=60,"P39",IF(AG43&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF43&lt;7,"À rechercher",IF(AG43&gt;=75,"P1",IF(AG43&gt;=60,"P2",IF(AG43&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI43" s="31"/>
@@ -4137,7 +4171,7 @@
         <x:f>IF(AF44&gt;=7,SUM(V44:AE44),"")</x:f>
       </x:c>
       <x:c r="AH44" s="33" t="str">
-        <x:f>IF(AF44&lt;7,"À rechercher",IF(AG44&gt;=75,"P39",IF(AG44&gt;=60,"P40",IF(AG44&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF44&lt;7,"À rechercher",IF(AG44&gt;=75,"P1",IF(AG44&gt;=60,"P2",IF(AG44&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI44" s="31"/>
@@ -4208,7 +4242,7 @@
         <x:f>IF(AF45&gt;=7,SUM(V45:AE45),"")</x:f>
       </x:c>
       <x:c r="AH45" s="33" t="str">
-        <x:f>IF(AF45&lt;7,"À rechercher",IF(AG45&gt;=75,"P40",IF(AG45&gt;=60,"P41",IF(AG45&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF45&lt;7,"À rechercher",IF(AG45&gt;=75,"P1",IF(AG45&gt;=60,"P2",IF(AG45&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI45" s="31"/>
@@ -4279,7 +4313,7 @@
         <x:f>IF(AF46&gt;=7,SUM(V46:AE46),"")</x:f>
       </x:c>
       <x:c r="AH46" s="33" t="str">
-        <x:f>IF(AF46&lt;7,"À rechercher",IF(AG46&gt;=75,"P41",IF(AG46&gt;=60,"P42",IF(AG46&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF46&lt;7,"À rechercher",IF(AG46&gt;=75,"P1",IF(AG46&gt;=60,"P2",IF(AG46&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI46" s="31"/>
@@ -4350,7 +4384,7 @@
         <x:f>IF(AF47&gt;=7,SUM(V47:AE47),"")</x:f>
       </x:c>
       <x:c r="AH47" s="33" t="str">
-        <x:f>IF(AF47&lt;7,"À rechercher",IF(AG47&gt;=75,"P42",IF(AG47&gt;=60,"P43",IF(AG47&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF47&lt;7,"À rechercher",IF(AG47&gt;=75,"P1",IF(AG47&gt;=60,"P2",IF(AG47&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI47" s="31"/>
@@ -4421,7 +4455,7 @@
         <x:f>IF(AF48&gt;=7,SUM(V48:AE48),"")</x:f>
       </x:c>
       <x:c r="AH48" s="33" t="str">
-        <x:f>IF(AF48&lt;7,"À rechercher",IF(AG48&gt;=75,"P43",IF(AG48&gt;=60,"P44",IF(AG48&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF48&lt;7,"À rechercher",IF(AG48&gt;=75,"P1",IF(AG48&gt;=60,"P2",IF(AG48&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI48" s="31"/>
@@ -4492,7 +4526,7 @@
         <x:f>IF(AF49&gt;=7,SUM(V49:AE49),"")</x:f>
       </x:c>
       <x:c r="AH49" s="33" t="str">
-        <x:f>IF(AF49&lt;7,"À rechercher",IF(AG49&gt;=75,"P44",IF(AG49&gt;=60,"P45",IF(AG49&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF49&lt;7,"À rechercher",IF(AG49&gt;=75,"P1",IF(AG49&gt;=60,"P2",IF(AG49&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI49" s="31"/>
@@ -4563,7 +4597,7 @@
         <x:f>IF(AF50&gt;=7,SUM(V50:AE50),"")</x:f>
       </x:c>
       <x:c r="AH50" s="33" t="str">
-        <x:f>IF(AF50&lt;7,"À rechercher",IF(AG50&gt;=75,"P45",IF(AG50&gt;=60,"P46",IF(AG50&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF50&lt;7,"À rechercher",IF(AG50&gt;=75,"P1",IF(AG50&gt;=60,"P2",IF(AG50&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI50" s="31"/>
@@ -4634,7 +4668,7 @@
         <x:f>IF(AF51&gt;=7,SUM(V51:AE51),"")</x:f>
       </x:c>
       <x:c r="AH51" s="33" t="str">
-        <x:f>IF(AF51&lt;7,"À rechercher",IF(AG51&gt;=75,"P46",IF(AG51&gt;=60,"P47",IF(AG51&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF51&lt;7,"À rechercher",IF(AG51&gt;=75,"P1",IF(AG51&gt;=60,"P2",IF(AG51&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI51" s="31"/>
@@ -4705,7 +4739,7 @@
         <x:f>IF(AF52&gt;=7,SUM(V52:AE52),"")</x:f>
       </x:c>
       <x:c r="AH52" s="33" t="str">
-        <x:f>IF(AF52&lt;7,"À rechercher",IF(AG52&gt;=75,"P47",IF(AG52&gt;=60,"P48",IF(AG52&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF52&lt;7,"À rechercher",IF(AG52&gt;=75,"P1",IF(AG52&gt;=60,"P2",IF(AG52&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI52" s="31"/>
@@ -4776,7 +4810,7 @@
         <x:f>IF(AF53&gt;=7,SUM(V53:AE53),"")</x:f>
       </x:c>
       <x:c r="AH53" s="33" t="str">
-        <x:f>IF(AF53&lt;7,"À rechercher",IF(AG53&gt;=75,"P48",IF(AG53&gt;=60,"P49",IF(AG53&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF53&lt;7,"À rechercher",IF(AG53&gt;=75,"P1",IF(AG53&gt;=60,"P2",IF(AG53&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI53" s="31"/>
@@ -4847,7 +4881,7 @@
         <x:f>IF(AF54&gt;=7,SUM(V54:AE54),"")</x:f>
       </x:c>
       <x:c r="AH54" s="33" t="str">
-        <x:f>IF(AF54&lt;7,"À rechercher",IF(AG54&gt;=75,"P49",IF(AG54&gt;=60,"P50",IF(AG54&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF54&lt;7,"À rechercher",IF(AG54&gt;=75,"P1",IF(AG54&gt;=60,"P2",IF(AG54&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI54" s="31"/>
@@ -4918,7 +4952,7 @@
         <x:f>IF(AF55&gt;=7,SUM(V55:AE55),"")</x:f>
       </x:c>
       <x:c r="AH55" s="33" t="str">
-        <x:f>IF(AF55&lt;7,"À rechercher",IF(AG55&gt;=75,"P50",IF(AG55&gt;=60,"P51",IF(AG55&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF55&lt;7,"À rechercher",IF(AG55&gt;=75,"P1",IF(AG55&gt;=60,"P2",IF(AG55&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI55" s="31"/>
@@ -4989,7 +5023,7 @@
         <x:f>IF(AF56&gt;=7,SUM(V56:AE56),"")</x:f>
       </x:c>
       <x:c r="AH56" s="33" t="str">
-        <x:f>IF(AF56&lt;7,"À rechercher",IF(AG56&gt;=75,"P51",IF(AG56&gt;=60,"P52",IF(AG56&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF56&lt;7,"À rechercher",IF(AG56&gt;=75,"P1",IF(AG56&gt;=60,"P2",IF(AG56&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI56" s="31"/>
@@ -5060,7 +5094,7 @@
         <x:f>IF(AF57&gt;=7,SUM(V57:AE57),"")</x:f>
       </x:c>
       <x:c r="AH57" s="33" t="str">
-        <x:f>IF(AF57&lt;7,"À rechercher",IF(AG57&gt;=75,"P52",IF(AG57&gt;=60,"P53",IF(AG57&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF57&lt;7,"À rechercher",IF(AG57&gt;=75,"P1",IF(AG57&gt;=60,"P2",IF(AG57&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI57" s="31"/>
@@ -5131,7 +5165,7 @@
         <x:f>IF(AF58&gt;=7,SUM(V58:AE58),"")</x:f>
       </x:c>
       <x:c r="AH58" s="33" t="str">
-        <x:f>IF(AF58&lt;7,"À rechercher",IF(AG58&gt;=75,"P53",IF(AG58&gt;=60,"P54",IF(AG58&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF58&lt;7,"À rechercher",IF(AG58&gt;=75,"P1",IF(AG58&gt;=60,"P2",IF(AG58&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI58" s="31"/>
@@ -5202,7 +5236,7 @@
         <x:f>IF(AF59&gt;=7,SUM(V59:AE59),"")</x:f>
       </x:c>
       <x:c r="AH59" s="33" t="str">
-        <x:f>IF(AF59&lt;7,"À rechercher",IF(AG59&gt;=75,"P54",IF(AG59&gt;=60,"P55",IF(AG59&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF59&lt;7,"À rechercher",IF(AG59&gt;=75,"P1",IF(AG59&gt;=60,"P2",IF(AG59&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI59" s="31"/>
@@ -5273,7 +5307,7 @@
         <x:f>IF(AF60&gt;=7,SUM(V60:AE60),"")</x:f>
       </x:c>
       <x:c r="AH60" s="33" t="str">
-        <x:f>IF(AF60&lt;7,"À rechercher",IF(AG60&gt;=75,"P55",IF(AG60&gt;=60,"P56",IF(AG60&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF60&lt;7,"À rechercher",IF(AG60&gt;=75,"P1",IF(AG60&gt;=60,"P2",IF(AG60&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI60" s="31"/>
@@ -5344,7 +5378,7 @@
         <x:f>IF(AF61&gt;=7,SUM(V61:AE61),"")</x:f>
       </x:c>
       <x:c r="AH61" s="33" t="str">
-        <x:f>IF(AF61&lt;7,"À rechercher",IF(AG61&gt;=75,"P56",IF(AG61&gt;=60,"P57",IF(AG61&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF61&lt;7,"À rechercher",IF(AG61&gt;=75,"P1",IF(AG61&gt;=60,"P2",IF(AG61&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI61" s="31"/>
@@ -5415,7 +5449,7 @@
         <x:f>IF(AF62&gt;=7,SUM(V62:AE62),"")</x:f>
       </x:c>
       <x:c r="AH62" s="33" t="str">
-        <x:f>IF(AF62&lt;7,"À rechercher",IF(AG62&gt;=75,"P57",IF(AG62&gt;=60,"P58",IF(AG62&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF62&lt;7,"À rechercher",IF(AG62&gt;=75,"P1",IF(AG62&gt;=60,"P2",IF(AG62&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI62" s="31"/>
@@ -5486,7 +5520,7 @@
         <x:f>IF(AF63&gt;=7,SUM(V63:AE63),"")</x:f>
       </x:c>
       <x:c r="AH63" s="33" t="str">
-        <x:f>IF(AF63&lt;7,"À rechercher",IF(AG63&gt;=75,"P58",IF(AG63&gt;=60,"P59",IF(AG63&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF63&lt;7,"À rechercher",IF(AG63&gt;=75,"P1",IF(AG63&gt;=60,"P2",IF(AG63&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI63" s="31"/>
@@ -5557,7 +5591,7 @@
         <x:f>IF(AF64&gt;=7,SUM(V64:AE64),"")</x:f>
       </x:c>
       <x:c r="AH64" s="33" t="str">
-        <x:f>IF(AF64&lt;7,"À rechercher",IF(AG64&gt;=75,"P59",IF(AG64&gt;=60,"P60",IF(AG64&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF64&lt;7,"À rechercher",IF(AG64&gt;=75,"P1",IF(AG64&gt;=60,"P2",IF(AG64&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI64" s="31"/>
@@ -5628,7 +5662,7 @@
         <x:f>IF(AF65&gt;=7,SUM(V65:AE65),"")</x:f>
       </x:c>
       <x:c r="AH65" s="33" t="str">
-        <x:f>IF(AF65&lt;7,"À rechercher",IF(AG65&gt;=75,"P60",IF(AG65&gt;=60,"P61",IF(AG65&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF65&lt;7,"À rechercher",IF(AG65&gt;=75,"P1",IF(AG65&gt;=60,"P2",IF(AG65&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI65" s="31"/>
@@ -5699,7 +5733,7 @@
         <x:f>IF(AF66&gt;=7,SUM(V66:AE66),"")</x:f>
       </x:c>
       <x:c r="AH66" s="33" t="str">
-        <x:f>IF(AF66&lt;7,"À rechercher",IF(AG66&gt;=75,"P61",IF(AG66&gt;=60,"P62",IF(AG66&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF66&lt;7,"À rechercher",IF(AG66&gt;=75,"P1",IF(AG66&gt;=60,"P2",IF(AG66&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI66" s="31"/>
@@ -5770,7 +5804,7 @@
         <x:f>IF(AF67&gt;=7,SUM(V67:AE67),"")</x:f>
       </x:c>
       <x:c r="AH67" s="33" t="str">
-        <x:f>IF(AF67&lt;7,"À rechercher",IF(AG67&gt;=75,"P62",IF(AG67&gt;=60,"P63",IF(AG67&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF67&lt;7,"À rechercher",IF(AG67&gt;=75,"P1",IF(AG67&gt;=60,"P2",IF(AG67&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI67" s="31"/>
@@ -5841,7 +5875,7 @@
         <x:f>IF(AF68&gt;=7,SUM(V68:AE68),"")</x:f>
       </x:c>
       <x:c r="AH68" s="33" t="str">
-        <x:f>IF(AF68&lt;7,"À rechercher",IF(AG68&gt;=75,"P63",IF(AG68&gt;=60,"P64",IF(AG68&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF68&lt;7,"À rechercher",IF(AG68&gt;=75,"P1",IF(AG68&gt;=60,"P2",IF(AG68&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI68" s="31"/>
@@ -5912,7 +5946,7 @@
         <x:f>IF(AF69&gt;=7,SUM(V69:AE69),"")</x:f>
       </x:c>
       <x:c r="AH69" s="33" t="str">
-        <x:f>IF(AF69&lt;7,"À rechercher",IF(AG69&gt;=75,"P64",IF(AG69&gt;=60,"P65",IF(AG69&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF69&lt;7,"À rechercher",IF(AG69&gt;=75,"P1",IF(AG69&gt;=60,"P2",IF(AG69&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI69" s="31"/>
@@ -5983,7 +6017,7 @@
         <x:f>IF(AF70&gt;=7,SUM(V70:AE70),"")</x:f>
       </x:c>
       <x:c r="AH70" s="33" t="str">
-        <x:f>IF(AF70&lt;7,"À rechercher",IF(AG70&gt;=75,"P65",IF(AG70&gt;=60,"P66",IF(AG70&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF70&lt;7,"À rechercher",IF(AG70&gt;=75,"P1",IF(AG70&gt;=60,"P2",IF(AG70&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI70" s="31"/>
@@ -6054,7 +6088,7 @@
         <x:f>IF(AF71&gt;=7,SUM(V71:AE71),"")</x:f>
       </x:c>
       <x:c r="AH71" s="33" t="str">
-        <x:f>IF(AF71&lt;7,"À rechercher",IF(AG71&gt;=75,"P66",IF(AG71&gt;=60,"P67",IF(AG71&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF71&lt;7,"À rechercher",IF(AG71&gt;=75,"P1",IF(AG71&gt;=60,"P2",IF(AG71&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI71" s="31"/>
@@ -6125,7 +6159,7 @@
         <x:f>IF(AF72&gt;=7,SUM(V72:AE72),"")</x:f>
       </x:c>
       <x:c r="AH72" s="33" t="str">
-        <x:f>IF(AF72&lt;7,"À rechercher",IF(AG72&gt;=75,"P67",IF(AG72&gt;=60,"P68",IF(AG72&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF72&lt;7,"À rechercher",IF(AG72&gt;=75,"P1",IF(AG72&gt;=60,"P2",IF(AG72&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI72" s="31"/>
@@ -6196,7 +6230,7 @@
         <x:f>IF(AF73&gt;=7,SUM(V73:AE73),"")</x:f>
       </x:c>
       <x:c r="AH73" s="33" t="str">
-        <x:f>IF(AF73&lt;7,"À rechercher",IF(AG73&gt;=75,"P68",IF(AG73&gt;=60,"P69",IF(AG73&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF73&lt;7,"À rechercher",IF(AG73&gt;=75,"P1",IF(AG73&gt;=60,"P2",IF(AG73&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI73" s="31"/>
@@ -6267,7 +6301,7 @@
         <x:f>IF(AF74&gt;=7,SUM(V74:AE74),"")</x:f>
       </x:c>
       <x:c r="AH74" s="33" t="str">
-        <x:f>IF(AF74&lt;7,"À rechercher",IF(AG74&gt;=75,"P69",IF(AG74&gt;=60,"P70",IF(AG74&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF74&lt;7,"À rechercher",IF(AG74&gt;=75,"P1",IF(AG74&gt;=60,"P2",IF(AG74&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI74" s="31"/>
@@ -6338,7 +6372,7 @@
         <x:f>IF(AF75&gt;=7,SUM(V75:AE75),"")</x:f>
       </x:c>
       <x:c r="AH75" s="33" t="str">
-        <x:f>IF(AF75&lt;7,"À rechercher",IF(AG75&gt;=75,"P70",IF(AG75&gt;=60,"P71",IF(AG75&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF75&lt;7,"À rechercher",IF(AG75&gt;=75,"P1",IF(AG75&gt;=60,"P2",IF(AG75&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI75" s="31"/>
@@ -6409,7 +6443,7 @@
         <x:f>IF(AF76&gt;=7,SUM(V76:AE76),"")</x:f>
       </x:c>
       <x:c r="AH76" s="33" t="str">
-        <x:f>IF(AF76&lt;7,"À rechercher",IF(AG76&gt;=75,"P71",IF(AG76&gt;=60,"P72",IF(AG76&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF76&lt;7,"À rechercher",IF(AG76&gt;=75,"P1",IF(AG76&gt;=60,"P2",IF(AG76&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI76" s="31"/>
@@ -6480,7 +6514,7 @@
         <x:f>IF(AF77&gt;=7,SUM(V77:AE77),"")</x:f>
       </x:c>
       <x:c r="AH77" s="33" t="str">
-        <x:f>IF(AF77&lt;7,"À rechercher",IF(AG77&gt;=75,"P72",IF(AG77&gt;=60,"P73",IF(AG77&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF77&lt;7,"À rechercher",IF(AG77&gt;=75,"P1",IF(AG77&gt;=60,"P2",IF(AG77&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI77" s="31"/>
@@ -6551,7 +6585,7 @@
         <x:f>IF(AF78&gt;=7,SUM(V78:AE78),"")</x:f>
       </x:c>
       <x:c r="AH78" s="33" t="str">
-        <x:f>IF(AF78&lt;7,"À rechercher",IF(AG78&gt;=75,"P73",IF(AG78&gt;=60,"P74",IF(AG78&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF78&lt;7,"À rechercher",IF(AG78&gt;=75,"P1",IF(AG78&gt;=60,"P2",IF(AG78&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI78" s="31"/>
@@ -6622,7 +6656,7 @@
         <x:f>IF(AF79&gt;=7,SUM(V79:AE79),"")</x:f>
       </x:c>
       <x:c r="AH79" s="33" t="str">
-        <x:f>IF(AF79&lt;7,"À rechercher",IF(AG79&gt;=75,"P74",IF(AG79&gt;=60,"P75",IF(AG79&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF79&lt;7,"À rechercher",IF(AG79&gt;=75,"P1",IF(AG79&gt;=60,"P2",IF(AG79&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI79" s="31"/>
@@ -6693,7 +6727,7 @@
         <x:f>IF(AF80&gt;=7,SUM(V80:AE80),"")</x:f>
       </x:c>
       <x:c r="AH80" s="33" t="str">
-        <x:f>IF(AF80&lt;7,"À rechercher",IF(AG80&gt;=75,"P75",IF(AG80&gt;=60,"P76",IF(AG80&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF80&lt;7,"À rechercher",IF(AG80&gt;=75,"P1",IF(AG80&gt;=60,"P2",IF(AG80&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI80" s="31"/>
@@ -6764,7 +6798,7 @@
         <x:f>IF(AF81&gt;=7,SUM(V81:AE81),"")</x:f>
       </x:c>
       <x:c r="AH81" s="33" t="str">
-        <x:f>IF(AF81&lt;7,"À rechercher",IF(AG81&gt;=75,"P76",IF(AG81&gt;=60,"P77",IF(AG81&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF81&lt;7,"À rechercher",IF(AG81&gt;=75,"P1",IF(AG81&gt;=60,"P2",IF(AG81&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI81" s="31"/>
@@ -6835,7 +6869,7 @@
         <x:f>IF(AF82&gt;=7,SUM(V82:AE82),"")</x:f>
       </x:c>
       <x:c r="AH82" s="33" t="str">
-        <x:f>IF(AF82&lt;7,"À rechercher",IF(AG82&gt;=75,"P77",IF(AG82&gt;=60,"P78",IF(AG82&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF82&lt;7,"À rechercher",IF(AG82&gt;=75,"P1",IF(AG82&gt;=60,"P2",IF(AG82&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI82" s="31"/>
@@ -6906,7 +6940,7 @@
         <x:f>IF(AF83&gt;=7,SUM(V83:AE83),"")</x:f>
       </x:c>
       <x:c r="AH83" s="33" t="str">
-        <x:f>IF(AF83&lt;7,"À rechercher",IF(AG83&gt;=75,"P78",IF(AG83&gt;=60,"P79",IF(AG83&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF83&lt;7,"À rechercher",IF(AG83&gt;=75,"P1",IF(AG83&gt;=60,"P2",IF(AG83&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI83" s="31"/>
@@ -6977,7 +7011,7 @@
         <x:f>IF(AF84&gt;=7,SUM(V84:AE84),"")</x:f>
       </x:c>
       <x:c r="AH84" s="33" t="str">
-        <x:f>IF(AF84&lt;7,"À rechercher",IF(AG84&gt;=75,"P79",IF(AG84&gt;=60,"P80",IF(AG84&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF84&lt;7,"À rechercher",IF(AG84&gt;=75,"P1",IF(AG84&gt;=60,"P2",IF(AG84&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI84" s="31"/>
@@ -7048,7 +7082,7 @@
         <x:f>IF(AF85&gt;=7,SUM(V85:AE85),"")</x:f>
       </x:c>
       <x:c r="AH85" s="33" t="str">
-        <x:f>IF(AF85&lt;7,"À rechercher",IF(AG85&gt;=75,"P80",IF(AG85&gt;=60,"P81",IF(AG85&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF85&lt;7,"À rechercher",IF(AG85&gt;=75,"P1",IF(AG85&gt;=60,"P2",IF(AG85&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI85" s="31"/>
@@ -7119,7 +7153,7 @@
         <x:f>IF(AF86&gt;=7,SUM(V86:AE86),"")</x:f>
       </x:c>
       <x:c r="AH86" s="33" t="str">
-        <x:f>IF(AF86&lt;7,"À rechercher",IF(AG86&gt;=75,"P81",IF(AG86&gt;=60,"P82",IF(AG86&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF86&lt;7,"À rechercher",IF(AG86&gt;=75,"P1",IF(AG86&gt;=60,"P2",IF(AG86&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI86" s="31"/>
@@ -7190,7 +7224,7 @@
         <x:f>IF(AF87&gt;=7,SUM(V87:AE87),"")</x:f>
       </x:c>
       <x:c r="AH87" s="33" t="str">
-        <x:f>IF(AF87&lt;7,"À rechercher",IF(AG87&gt;=75,"P82",IF(AG87&gt;=60,"P83",IF(AG87&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF87&lt;7,"À rechercher",IF(AG87&gt;=75,"P1",IF(AG87&gt;=60,"P2",IF(AG87&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI87" s="31"/>
@@ -7261,7 +7295,7 @@
         <x:f>IF(AF88&gt;=7,SUM(V88:AE88),"")</x:f>
       </x:c>
       <x:c r="AH88" s="33" t="str">
-        <x:f>IF(AF88&lt;7,"À rechercher",IF(AG88&gt;=75,"P83",IF(AG88&gt;=60,"P84",IF(AG88&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF88&lt;7,"À rechercher",IF(AG88&gt;=75,"P1",IF(AG88&gt;=60,"P2",IF(AG88&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI88" s="31"/>
@@ -7332,7 +7366,7 @@
         <x:f>IF(AF89&gt;=7,SUM(V89:AE89),"")</x:f>
       </x:c>
       <x:c r="AH89" s="33" t="str">
-        <x:f>IF(AF89&lt;7,"À rechercher",IF(AG89&gt;=75,"P84",IF(AG89&gt;=60,"P85",IF(AG89&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF89&lt;7,"À rechercher",IF(AG89&gt;=75,"P1",IF(AG89&gt;=60,"P2",IF(AG89&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI89" s="31"/>
@@ -7403,7 +7437,7 @@
         <x:f>IF(AF90&gt;=7,SUM(V90:AE90),"")</x:f>
       </x:c>
       <x:c r="AH90" s="33" t="str">
-        <x:f>IF(AF90&lt;7,"À rechercher",IF(AG90&gt;=75,"P85",IF(AG90&gt;=60,"P86",IF(AG90&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF90&lt;7,"À rechercher",IF(AG90&gt;=75,"P1",IF(AG90&gt;=60,"P2",IF(AG90&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI90" s="31"/>
@@ -7474,7 +7508,7 @@
         <x:f>IF(AF91&gt;=7,SUM(V91:AE91),"")</x:f>
       </x:c>
       <x:c r="AH91" s="33" t="str">
-        <x:f>IF(AF91&lt;7,"À rechercher",IF(AG91&gt;=75,"P86",IF(AG91&gt;=60,"P87",IF(AG91&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF91&lt;7,"À rechercher",IF(AG91&gt;=75,"P1",IF(AG91&gt;=60,"P2",IF(AG91&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI91" s="31"/>
@@ -7545,7 +7579,7 @@
         <x:f>IF(AF92&gt;=7,SUM(V92:AE92),"")</x:f>
       </x:c>
       <x:c r="AH92" s="33" t="str">
-        <x:f>IF(AF92&lt;7,"À rechercher",IF(AG92&gt;=75,"P87",IF(AG92&gt;=60,"P88",IF(AG92&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF92&lt;7,"À rechercher",IF(AG92&gt;=75,"P1",IF(AG92&gt;=60,"P2",IF(AG92&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI92" s="31"/>
@@ -7616,7 +7650,7 @@
         <x:f>IF(AF93&gt;=7,SUM(V93:AE93),"")</x:f>
       </x:c>
       <x:c r="AH93" s="33" t="str">
-        <x:f>IF(AF93&lt;7,"À rechercher",IF(AG93&gt;=75,"P88",IF(AG93&gt;=60,"P89",IF(AG93&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF93&lt;7,"À rechercher",IF(AG93&gt;=75,"P1",IF(AG93&gt;=60,"P2",IF(AG93&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI93" s="31"/>
@@ -7687,7 +7721,7 @@
         <x:f>IF(AF94&gt;=7,SUM(V94:AE94),"")</x:f>
       </x:c>
       <x:c r="AH94" s="33" t="str">
-        <x:f>IF(AF94&lt;7,"À rechercher",IF(AG94&gt;=75,"P89",IF(AG94&gt;=60,"P90",IF(AG94&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF94&lt;7,"À rechercher",IF(AG94&gt;=75,"P1",IF(AG94&gt;=60,"P2",IF(AG94&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI94" s="31"/>
@@ -7758,7 +7792,7 @@
         <x:f>IF(AF95&gt;=7,SUM(V95:AE95),"")</x:f>
       </x:c>
       <x:c r="AH95" s="33" t="str">
-        <x:f>IF(AF95&lt;7,"À rechercher",IF(AG95&gt;=75,"P90",IF(AG95&gt;=60,"P91",IF(AG95&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF95&lt;7,"À rechercher",IF(AG95&gt;=75,"P1",IF(AG95&gt;=60,"P2",IF(AG95&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI95" s="31"/>
@@ -7829,7 +7863,7 @@
         <x:f>IF(AF96&gt;=7,SUM(V96:AE96),"")</x:f>
       </x:c>
       <x:c r="AH96" s="33" t="str">
-        <x:f>IF(AF96&lt;7,"À rechercher",IF(AG96&gt;=75,"P91",IF(AG96&gt;=60,"P92",IF(AG96&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF96&lt;7,"À rechercher",IF(AG96&gt;=75,"P1",IF(AG96&gt;=60,"P2",IF(AG96&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI96" s="31"/>
@@ -7900,7 +7934,7 @@
         <x:f>IF(AF97&gt;=7,SUM(V97:AE97),"")</x:f>
       </x:c>
       <x:c r="AH97" s="33" t="str">
-        <x:f>IF(AF97&lt;7,"À rechercher",IF(AG97&gt;=75,"P92",IF(AG97&gt;=60,"P93",IF(AG97&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF97&lt;7,"À rechercher",IF(AG97&gt;=75,"P1",IF(AG97&gt;=60,"P2",IF(AG97&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI97" s="31"/>
@@ -7971,7 +8005,7 @@
         <x:f>IF(AF98&gt;=7,SUM(V98:AE98),"")</x:f>
       </x:c>
       <x:c r="AH98" s="33" t="str">
-        <x:f>IF(AF98&lt;7,"À rechercher",IF(AG98&gt;=75,"P93",IF(AG98&gt;=60,"P94",IF(AG98&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF98&lt;7,"À rechercher",IF(AG98&gt;=75,"P1",IF(AG98&gt;=60,"P2",IF(AG98&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI98" s="31"/>
@@ -8042,7 +8076,7 @@
         <x:f>IF(AF99&gt;=7,SUM(V99:AE99),"")</x:f>
       </x:c>
       <x:c r="AH99" s="33" t="str">
-        <x:f>IF(AF99&lt;7,"À rechercher",IF(AG99&gt;=75,"P94",IF(AG99&gt;=60,"P95",IF(AG99&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF99&lt;7,"À rechercher",IF(AG99&gt;=75,"P1",IF(AG99&gt;=60,"P2",IF(AG99&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI99" s="31"/>
@@ -8113,7 +8147,7 @@
         <x:f>IF(AF100&gt;=7,SUM(V100:AE100),"")</x:f>
       </x:c>
       <x:c r="AH100" s="33" t="str">
-        <x:f>IF(AF100&lt;7,"À rechercher",IF(AG100&gt;=75,"P95",IF(AG100&gt;=60,"P96",IF(AG100&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF100&lt;7,"À rechercher",IF(AG100&gt;=75,"P1",IF(AG100&gt;=60,"P2",IF(AG100&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI100" s="31"/>
@@ -8184,7 +8218,7 @@
         <x:f>IF(AF101&gt;=7,SUM(V101:AE101),"")</x:f>
       </x:c>
       <x:c r="AH101" s="33" t="str">
-        <x:f>IF(AF101&lt;7,"À rechercher",IF(AG101&gt;=75,"P96",IF(AG101&gt;=60,"P97",IF(AG101&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF101&lt;7,"À rechercher",IF(AG101&gt;=75,"P1",IF(AG101&gt;=60,"P2",IF(AG101&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI101" s="31"/>
@@ -8255,7 +8289,7 @@
         <x:f>IF(AF102&gt;=7,SUM(V102:AE102),"")</x:f>
       </x:c>
       <x:c r="AH102" s="33" t="str">
-        <x:f>IF(AF102&lt;7,"À rechercher",IF(AG102&gt;=75,"P97",IF(AG102&gt;=60,"P98",IF(AG102&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF102&lt;7,"À rechercher",IF(AG102&gt;=75,"P1",IF(AG102&gt;=60,"P2",IF(AG102&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI102" s="31"/>
@@ -8326,7 +8360,7 @@
         <x:f>IF(AF103&gt;=7,SUM(V103:AE103),"")</x:f>
       </x:c>
       <x:c r="AH103" s="33" t="str">
-        <x:f>IF(AF103&lt;7,"À rechercher",IF(AG103&gt;=75,"P98",IF(AG103&gt;=60,"P99",IF(AG103&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF103&lt;7,"À rechercher",IF(AG103&gt;=75,"P1",IF(AG103&gt;=60,"P2",IF(AG103&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI103" s="31"/>
@@ -8397,7 +8431,7 @@
         <x:f>IF(AF104&gt;=7,SUM(V104:AE104),"")</x:f>
       </x:c>
       <x:c r="AH104" s="33" t="str">
-        <x:f>IF(AF104&lt;7,"À rechercher",IF(AG104&gt;=75,"P99",IF(AG104&gt;=60,"P100",IF(AG104&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF104&lt;7,"À rechercher",IF(AG104&gt;=75,"P1",IF(AG104&gt;=60,"P2",IF(AG104&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI104" s="31"/>
@@ -8468,7 +8502,7 @@
         <x:f>IF(AF105&gt;=7,SUM(V105:AE105),"")</x:f>
       </x:c>
       <x:c r="AH105" s="33" t="str">
-        <x:f>IF(AF105&lt;7,"À rechercher",IF(AG105&gt;=75,"P100",IF(AG105&gt;=60,"P101",IF(AG105&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF105&lt;7,"À rechercher",IF(AG105&gt;=75,"P1",IF(AG105&gt;=60,"P2",IF(AG105&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI105" s="31"/>
@@ -8539,7 +8573,7 @@
         <x:f>IF(AF106&gt;=7,SUM(V106:AE106),"")</x:f>
       </x:c>
       <x:c r="AH106" s="33" t="str">
-        <x:f>IF(AF106&lt;7,"À rechercher",IF(AG106&gt;=75,"P101",IF(AG106&gt;=60,"P102",IF(AG106&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF106&lt;7,"À rechercher",IF(AG106&gt;=75,"P1",IF(AG106&gt;=60,"P2",IF(AG106&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI106" s="31"/>
@@ -8610,7 +8644,7 @@
         <x:f>IF(AF107&gt;=7,SUM(V107:AE107),"")</x:f>
       </x:c>
       <x:c r="AH107" s="33" t="str">
-        <x:f>IF(AF107&lt;7,"À rechercher",IF(AG107&gt;=75,"P102",IF(AG107&gt;=60,"P103",IF(AG107&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF107&lt;7,"À rechercher",IF(AG107&gt;=75,"P1",IF(AG107&gt;=60,"P2",IF(AG107&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI107" s="31"/>
@@ -8681,7 +8715,7 @@
         <x:f>IF(AF108&gt;=7,SUM(V108:AE108),"")</x:f>
       </x:c>
       <x:c r="AH108" s="33" t="str">
-        <x:f>IF(AF108&lt;7,"À rechercher",IF(AG108&gt;=75,"P103",IF(AG108&gt;=60,"P104",IF(AG108&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF108&lt;7,"À rechercher",IF(AG108&gt;=75,"P1",IF(AG108&gt;=60,"P2",IF(AG108&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI108" s="31"/>
@@ -8752,7 +8786,7 @@
         <x:f>IF(AF109&gt;=7,SUM(V109:AE109),"")</x:f>
       </x:c>
       <x:c r="AH109" s="33" t="str">
-        <x:f>IF(AF109&lt;7,"À rechercher",IF(AG109&gt;=75,"P104",IF(AG109&gt;=60,"P105",IF(AG109&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF109&lt;7,"À rechercher",IF(AG109&gt;=75,"P1",IF(AG109&gt;=60,"P2",IF(AG109&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI109" s="31"/>
@@ -8823,7 +8857,7 @@
         <x:f>IF(AF110&gt;=7,SUM(V110:AE110),"")</x:f>
       </x:c>
       <x:c r="AH110" s="33" t="str">
-        <x:f>IF(AF110&lt;7,"À rechercher",IF(AG110&gt;=75,"P105",IF(AG110&gt;=60,"P106",IF(AG110&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF110&lt;7,"À rechercher",IF(AG110&gt;=75,"P1",IF(AG110&gt;=60,"P2",IF(AG110&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI110" s="31"/>
@@ -8894,7 +8928,7 @@
         <x:f>IF(AF111&gt;=7,SUM(V111:AE111),"")</x:f>
       </x:c>
       <x:c r="AH111" s="33" t="str">
-        <x:f>IF(AF111&lt;7,"À rechercher",IF(AG111&gt;=75,"P106",IF(AG111&gt;=60,"P107",IF(AG111&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF111&lt;7,"À rechercher",IF(AG111&gt;=75,"P1",IF(AG111&gt;=60,"P2",IF(AG111&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI111" s="31"/>
@@ -8965,7 +8999,7 @@
         <x:f>IF(AF112&gt;=7,SUM(V112:AE112),"")</x:f>
       </x:c>
       <x:c r="AH112" s="33" t="str">
-        <x:f>IF(AF112&lt;7,"À rechercher",IF(AG112&gt;=75,"P107",IF(AG112&gt;=60,"P108",IF(AG112&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF112&lt;7,"À rechercher",IF(AG112&gt;=75,"P1",IF(AG112&gt;=60,"P2",IF(AG112&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI112" s="31"/>
@@ -9036,7 +9070,7 @@
         <x:f>IF(AF113&gt;=7,SUM(V113:AE113),"")</x:f>
       </x:c>
       <x:c r="AH113" s="33" t="str">
-        <x:f>IF(AF113&lt;7,"À rechercher",IF(AG113&gt;=75,"P108",IF(AG113&gt;=60,"P109",IF(AG113&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF113&lt;7,"À rechercher",IF(AG113&gt;=75,"P1",IF(AG113&gt;=60,"P2",IF(AG113&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI113" s="31"/>
@@ -9107,7 +9141,7 @@
         <x:f>IF(AF114&gt;=7,SUM(V114:AE114),"")</x:f>
       </x:c>
       <x:c r="AH114" s="33" t="str">
-        <x:f>IF(AF114&lt;7,"À rechercher",IF(AG114&gt;=75,"P109",IF(AG114&gt;=60,"P110",IF(AG114&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF114&lt;7,"À rechercher",IF(AG114&gt;=75,"P1",IF(AG114&gt;=60,"P2",IF(AG114&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI114" s="31"/>
@@ -9178,7 +9212,7 @@
         <x:f>IF(AF115&gt;=7,SUM(V115:AE115),"")</x:f>
       </x:c>
       <x:c r="AH115" s="33" t="str">
-        <x:f>IF(AF115&lt;7,"À rechercher",IF(AG115&gt;=75,"P110",IF(AG115&gt;=60,"P111",IF(AG115&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF115&lt;7,"À rechercher",IF(AG115&gt;=75,"P1",IF(AG115&gt;=60,"P2",IF(AG115&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI115" s="31"/>
@@ -9249,7 +9283,7 @@
         <x:f>IF(AF116&gt;=7,SUM(V116:AE116),"")</x:f>
       </x:c>
       <x:c r="AH116" s="33" t="str">
-        <x:f>IF(AF116&lt;7,"À rechercher",IF(AG116&gt;=75,"P111",IF(AG116&gt;=60,"P112",IF(AG116&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF116&lt;7,"À rechercher",IF(AG116&gt;=75,"P1",IF(AG116&gt;=60,"P2",IF(AG116&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI116" s="31"/>
@@ -9320,7 +9354,7 @@
         <x:f>IF(AF117&gt;=7,SUM(V117:AE117),"")</x:f>
       </x:c>
       <x:c r="AH117" s="33" t="str">
-        <x:f>IF(AF117&lt;7,"À rechercher",IF(AG117&gt;=75,"P112",IF(AG117&gt;=60,"P113",IF(AG117&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF117&lt;7,"À rechercher",IF(AG117&gt;=75,"P1",IF(AG117&gt;=60,"P2",IF(AG117&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI117" s="31"/>
@@ -9391,7 +9425,7 @@
         <x:f>IF(AF118&gt;=7,SUM(V118:AE118),"")</x:f>
       </x:c>
       <x:c r="AH118" s="33" t="str">
-        <x:f>IF(AF118&lt;7,"À rechercher",IF(AG118&gt;=75,"P113",IF(AG118&gt;=60,"P114",IF(AG118&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF118&lt;7,"À rechercher",IF(AG118&gt;=75,"P1",IF(AG118&gt;=60,"P2",IF(AG118&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI118" s="31"/>
@@ -9462,7 +9496,7 @@
         <x:f>IF(AF119&gt;=7,SUM(V119:AE119),"")</x:f>
       </x:c>
       <x:c r="AH119" s="33" t="str">
-        <x:f>IF(AF119&lt;7,"À rechercher",IF(AG119&gt;=75,"P114",IF(AG119&gt;=60,"P115",IF(AG119&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF119&lt;7,"À rechercher",IF(AG119&gt;=75,"P1",IF(AG119&gt;=60,"P2",IF(AG119&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI119" s="31"/>
@@ -9533,7 +9567,7 @@
         <x:f>IF(AF120&gt;=7,SUM(V120:AE120),"")</x:f>
       </x:c>
       <x:c r="AH120" s="33" t="str">
-        <x:f>IF(AF120&lt;7,"À rechercher",IF(AG120&gt;=75,"P115",IF(AG120&gt;=60,"P116",IF(AG120&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF120&lt;7,"À rechercher",IF(AG120&gt;=75,"P1",IF(AG120&gt;=60,"P2",IF(AG120&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI120" s="31"/>
@@ -9604,7 +9638,7 @@
         <x:f>IF(AF121&gt;=7,SUM(V121:AE121),"")</x:f>
       </x:c>
       <x:c r="AH121" s="33" t="str">
-        <x:f>IF(AF121&lt;7,"À rechercher",IF(AG121&gt;=75,"P116",IF(AG121&gt;=60,"P117",IF(AG121&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF121&lt;7,"À rechercher",IF(AG121&gt;=75,"P1",IF(AG121&gt;=60,"P2",IF(AG121&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI121" s="31"/>
@@ -9675,7 +9709,7 @@
         <x:f>IF(AF122&gt;=7,SUM(V122:AE122),"")</x:f>
       </x:c>
       <x:c r="AH122" s="33" t="str">
-        <x:f>IF(AF122&lt;7,"À rechercher",IF(AG122&gt;=75,"P117",IF(AG122&gt;=60,"P118",IF(AG122&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF122&lt;7,"À rechercher",IF(AG122&gt;=75,"P1",IF(AG122&gt;=60,"P2",IF(AG122&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI122" s="31"/>
@@ -9746,7 +9780,7 @@
         <x:f>IF(AF123&gt;=7,SUM(V123:AE123),"")</x:f>
       </x:c>
       <x:c r="AH123" s="33" t="str">
-        <x:f>IF(AF123&lt;7,"À rechercher",IF(AG123&gt;=75,"P118",IF(AG123&gt;=60,"P119",IF(AG123&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF123&lt;7,"À rechercher",IF(AG123&gt;=75,"P1",IF(AG123&gt;=60,"P2",IF(AG123&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI123" s="31"/>
@@ -9817,7 +9851,7 @@
         <x:f>IF(AF124&gt;=7,SUM(V124:AE124),"")</x:f>
       </x:c>
       <x:c r="AH124" s="33" t="str">
-        <x:f>IF(AF124&lt;7,"À rechercher",IF(AG124&gt;=75,"P119",IF(AG124&gt;=60,"P120",IF(AG124&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF124&lt;7,"À rechercher",IF(AG124&gt;=75,"P1",IF(AG124&gt;=60,"P2",IF(AG124&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI124" s="31"/>
@@ -9888,7 +9922,7 @@
         <x:f>IF(AF125&gt;=7,SUM(V125:AE125),"")</x:f>
       </x:c>
       <x:c r="AH125" s="33" t="str">
-        <x:f>IF(AF125&lt;7,"À rechercher",IF(AG125&gt;=75,"P120",IF(AG125&gt;=60,"P121",IF(AG125&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF125&lt;7,"À rechercher",IF(AG125&gt;=75,"P1",IF(AG125&gt;=60,"P2",IF(AG125&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI125" s="31"/>
@@ -9959,7 +9993,7 @@
         <x:f>IF(AF126&gt;=7,SUM(V126:AE126),"")</x:f>
       </x:c>
       <x:c r="AH126" s="33" t="str">
-        <x:f>IF(AF126&lt;7,"À rechercher",IF(AG126&gt;=75,"P121",IF(AG126&gt;=60,"P122",IF(AG126&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF126&lt;7,"À rechercher",IF(AG126&gt;=75,"P1",IF(AG126&gt;=60,"P2",IF(AG126&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI126" s="31"/>
@@ -10030,7 +10064,7 @@
         <x:f>IF(AF127&gt;=7,SUM(V127:AE127),"")</x:f>
       </x:c>
       <x:c r="AH127" s="33" t="str">
-        <x:f>IF(AF127&lt;7,"À rechercher",IF(AG127&gt;=75,"P122",IF(AG127&gt;=60,"P123",IF(AG127&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF127&lt;7,"À rechercher",IF(AG127&gt;=75,"P1",IF(AG127&gt;=60,"P2",IF(AG127&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI127" s="31"/>
@@ -10101,7 +10135,7 @@
         <x:f>IF(AF128&gt;=7,SUM(V128:AE128),"")</x:f>
       </x:c>
       <x:c r="AH128" s="33" t="str">
-        <x:f>IF(AF128&lt;7,"À rechercher",IF(AG128&gt;=75,"P123",IF(AG128&gt;=60,"P124",IF(AG128&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF128&lt;7,"À rechercher",IF(AG128&gt;=75,"P1",IF(AG128&gt;=60,"P2",IF(AG128&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI128" s="31"/>
@@ -10172,7 +10206,7 @@
         <x:f>IF(AF129&gt;=7,SUM(V129:AE129),"")</x:f>
       </x:c>
       <x:c r="AH129" s="33" t="str">
-        <x:f>IF(AF129&lt;7,"À rechercher",IF(AG129&gt;=75,"P124",IF(AG129&gt;=60,"P125",IF(AG129&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF129&lt;7,"À rechercher",IF(AG129&gt;=75,"P1",IF(AG129&gt;=60,"P2",IF(AG129&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI129" s="31"/>
@@ -10243,7 +10277,7 @@
         <x:f>IF(AF130&gt;=7,SUM(V130:AE130),"")</x:f>
       </x:c>
       <x:c r="AH130" s="33" t="str">
-        <x:f>IF(AF130&lt;7,"À rechercher",IF(AG130&gt;=75,"P125",IF(AG130&gt;=60,"P126",IF(AG130&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF130&lt;7,"À rechercher",IF(AG130&gt;=75,"P1",IF(AG130&gt;=60,"P2",IF(AG130&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI130" s="31"/>
@@ -10314,7 +10348,7 @@
         <x:f>IF(AF131&gt;=7,SUM(V131:AE131),"")</x:f>
       </x:c>
       <x:c r="AH131" s="33" t="str">
-        <x:f>IF(AF131&lt;7,"À rechercher",IF(AG131&gt;=75,"P126",IF(AG131&gt;=60,"P127",IF(AG131&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF131&lt;7,"À rechercher",IF(AG131&gt;=75,"P1",IF(AG131&gt;=60,"P2",IF(AG131&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI131" s="31"/>
@@ -10385,7 +10419,7 @@
         <x:f>IF(AF132&gt;=7,SUM(V132:AE132),"")</x:f>
       </x:c>
       <x:c r="AH132" s="33" t="str">
-        <x:f>IF(AF132&lt;7,"À rechercher",IF(AG132&gt;=75,"P127",IF(AG132&gt;=60,"P128",IF(AG132&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF132&lt;7,"À rechercher",IF(AG132&gt;=75,"P1",IF(AG132&gt;=60,"P2",IF(AG132&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI132" s="31"/>
@@ -10456,7 +10490,7 @@
         <x:f>IF(AF133&gt;=7,SUM(V133:AE133),"")</x:f>
       </x:c>
       <x:c r="AH133" s="33" t="str">
-        <x:f>IF(AF133&lt;7,"À rechercher",IF(AG133&gt;=75,"P128",IF(AG133&gt;=60,"P129",IF(AG133&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF133&lt;7,"À rechercher",IF(AG133&gt;=75,"P1",IF(AG133&gt;=60,"P2",IF(AG133&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI133" s="31"/>
@@ -10527,7 +10561,7 @@
         <x:f>IF(AF134&gt;=7,SUM(V134:AE134),"")</x:f>
       </x:c>
       <x:c r="AH134" s="33" t="str">
-        <x:f>IF(AF134&lt;7,"À rechercher",IF(AG134&gt;=75,"P129",IF(AG134&gt;=60,"P130",IF(AG134&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF134&lt;7,"À rechercher",IF(AG134&gt;=75,"P1",IF(AG134&gt;=60,"P2",IF(AG134&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI134" s="31"/>
@@ -10598,7 +10632,7 @@
         <x:f>IF(AF135&gt;=7,SUM(V135:AE135),"")</x:f>
       </x:c>
       <x:c r="AH135" s="33" t="str">
-        <x:f>IF(AF135&lt;7,"À rechercher",IF(AG135&gt;=75,"P130",IF(AG135&gt;=60,"P131",IF(AG135&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF135&lt;7,"À rechercher",IF(AG135&gt;=75,"P1",IF(AG135&gt;=60,"P2",IF(AG135&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI135" s="31"/>
@@ -10669,7 +10703,7 @@
         <x:f>IF(AF136&gt;=7,SUM(V136:AE136),"")</x:f>
       </x:c>
       <x:c r="AH136" s="33" t="str">
-        <x:f>IF(AF136&lt;7,"À rechercher",IF(AG136&gt;=75,"P131",IF(AG136&gt;=60,"P132",IF(AG136&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF136&lt;7,"À rechercher",IF(AG136&gt;=75,"P1",IF(AG136&gt;=60,"P2",IF(AG136&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI136" s="31"/>
@@ -10740,7 +10774,7 @@
         <x:f>IF(AF137&gt;=7,SUM(V137:AE137),"")</x:f>
       </x:c>
       <x:c r="AH137" s="33" t="str">
-        <x:f>IF(AF137&lt;7,"À rechercher",IF(AG137&gt;=75,"P132",IF(AG137&gt;=60,"P133",IF(AG137&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF137&lt;7,"À rechercher",IF(AG137&gt;=75,"P1",IF(AG137&gt;=60,"P2",IF(AG137&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI137" s="31"/>
@@ -10811,7 +10845,7 @@
         <x:f>IF(AF138&gt;=7,SUM(V138:AE138),"")</x:f>
       </x:c>
       <x:c r="AH138" s="33" t="str">
-        <x:f>IF(AF138&lt;7,"À rechercher",IF(AG138&gt;=75,"P133",IF(AG138&gt;=60,"P134",IF(AG138&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF138&lt;7,"À rechercher",IF(AG138&gt;=75,"P1",IF(AG138&gt;=60,"P2",IF(AG138&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI138" s="31"/>
@@ -10882,7 +10916,7 @@
         <x:f>IF(AF139&gt;=7,SUM(V139:AE139),"")</x:f>
       </x:c>
       <x:c r="AH139" s="33" t="str">
-        <x:f>IF(AF139&lt;7,"À rechercher",IF(AG139&gt;=75,"P134",IF(AG139&gt;=60,"P135",IF(AG139&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF139&lt;7,"À rechercher",IF(AG139&gt;=75,"P1",IF(AG139&gt;=60,"P2",IF(AG139&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI139" s="31"/>
@@ -10953,7 +10987,7 @@
         <x:f>IF(AF140&gt;=7,SUM(V140:AE140),"")</x:f>
       </x:c>
       <x:c r="AH140" s="33" t="str">
-        <x:f>IF(AF140&lt;7,"À rechercher",IF(AG140&gt;=75,"P135",IF(AG140&gt;=60,"P136",IF(AG140&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF140&lt;7,"À rechercher",IF(AG140&gt;=75,"P1",IF(AG140&gt;=60,"P2",IF(AG140&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI140" s="31"/>
@@ -11024,7 +11058,7 @@
         <x:f>IF(AF141&gt;=7,SUM(V141:AE141),"")</x:f>
       </x:c>
       <x:c r="AH141" s="33" t="str">
-        <x:f>IF(AF141&lt;7,"À rechercher",IF(AG141&gt;=75,"P136",IF(AG141&gt;=60,"P137",IF(AG141&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF141&lt;7,"À rechercher",IF(AG141&gt;=75,"P1",IF(AG141&gt;=60,"P2",IF(AG141&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI141" s="31"/>
@@ -11095,7 +11129,7 @@
         <x:f>IF(AF142&gt;=7,SUM(V142:AE142),"")</x:f>
       </x:c>
       <x:c r="AH142" s="33" t="str">
-        <x:f>IF(AF142&lt;7,"À rechercher",IF(AG142&gt;=75,"P137",IF(AG142&gt;=60,"P138",IF(AG142&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF142&lt;7,"À rechercher",IF(AG142&gt;=75,"P1",IF(AG142&gt;=60,"P2",IF(AG142&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI142" s="31"/>
@@ -11166,7 +11200,7 @@
         <x:f>IF(AF143&gt;=7,SUM(V143:AE143),"")</x:f>
       </x:c>
       <x:c r="AH143" s="33" t="str">
-        <x:f>IF(AF143&lt;7,"À rechercher",IF(AG143&gt;=75,"P138",IF(AG143&gt;=60,"P139",IF(AG143&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF143&lt;7,"À rechercher",IF(AG143&gt;=75,"P1",IF(AG143&gt;=60,"P2",IF(AG143&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI143" s="31"/>
@@ -11237,7 +11271,7 @@
         <x:f>IF(AF144&gt;=7,SUM(V144:AE144),"")</x:f>
       </x:c>
       <x:c r="AH144" s="33" t="str">
-        <x:f>IF(AF144&lt;7,"À rechercher",IF(AG144&gt;=75,"P139",IF(AG144&gt;=60,"P140",IF(AG144&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF144&lt;7,"À rechercher",IF(AG144&gt;=75,"P1",IF(AG144&gt;=60,"P2",IF(AG144&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI144" s="31"/>
@@ -11308,7 +11342,7 @@
         <x:f>IF(AF145&gt;=7,SUM(V145:AE145),"")</x:f>
       </x:c>
       <x:c r="AH145" s="33" t="str">
-        <x:f>IF(AF145&lt;7,"À rechercher",IF(AG145&gt;=75,"P140",IF(AG145&gt;=60,"P141",IF(AG145&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF145&lt;7,"À rechercher",IF(AG145&gt;=75,"P1",IF(AG145&gt;=60,"P2",IF(AG145&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI145" s="31"/>
@@ -11379,7 +11413,7 @@
         <x:f>IF(AF146&gt;=7,SUM(V146:AE146),"")</x:f>
       </x:c>
       <x:c r="AH146" s="33" t="str">
-        <x:f>IF(AF146&lt;7,"À rechercher",IF(AG146&gt;=75,"P141",IF(AG146&gt;=60,"P142",IF(AG146&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF146&lt;7,"À rechercher",IF(AG146&gt;=75,"P1",IF(AG146&gt;=60,"P2",IF(AG146&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI146" s="31"/>
@@ -11450,7 +11484,7 @@
         <x:f>IF(AF147&gt;=7,SUM(V147:AE147),"")</x:f>
       </x:c>
       <x:c r="AH147" s="33" t="str">
-        <x:f>IF(AF147&lt;7,"À rechercher",IF(AG147&gt;=75,"P142",IF(AG147&gt;=60,"P143",IF(AG147&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF147&lt;7,"À rechercher",IF(AG147&gt;=75,"P1",IF(AG147&gt;=60,"P2",IF(AG147&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI147" s="31"/>
@@ -11521,7 +11555,7 @@
         <x:f>IF(AF148&gt;=7,SUM(V148:AE148),"")</x:f>
       </x:c>
       <x:c r="AH148" s="33" t="str">
-        <x:f>IF(AF148&lt;7,"À rechercher",IF(AG148&gt;=75,"P143",IF(AG148&gt;=60,"P144",IF(AG148&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF148&lt;7,"À rechercher",IF(AG148&gt;=75,"P1",IF(AG148&gt;=60,"P2",IF(AG148&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI148" s="31"/>
@@ -11592,7 +11626,7 @@
         <x:f>IF(AF149&gt;=7,SUM(V149:AE149),"")</x:f>
       </x:c>
       <x:c r="AH149" s="33" t="str">
-        <x:f>IF(AF149&lt;7,"À rechercher",IF(AG149&gt;=75,"P144",IF(AG149&gt;=60,"P145",IF(AG149&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF149&lt;7,"À rechercher",IF(AG149&gt;=75,"P1",IF(AG149&gt;=60,"P2",IF(AG149&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI149" s="31"/>
@@ -11663,7 +11697,7 @@
         <x:f>IF(AF150&gt;=7,SUM(V150:AE150),"")</x:f>
       </x:c>
       <x:c r="AH150" s="33" t="str">
-        <x:f>IF(AF150&lt;7,"À rechercher",IF(AG150&gt;=75,"P145",IF(AG150&gt;=60,"P146",IF(AG150&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF150&lt;7,"À rechercher",IF(AG150&gt;=75,"P1",IF(AG150&gt;=60,"P2",IF(AG150&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI150" s="31"/>
@@ -11734,7 +11768,7 @@
         <x:f>IF(AF151&gt;=7,SUM(V151:AE151),"")</x:f>
       </x:c>
       <x:c r="AH151" s="33" t="str">
-        <x:f>IF(AF151&lt;7,"À rechercher",IF(AG151&gt;=75,"P146",IF(AG151&gt;=60,"P147",IF(AG151&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF151&lt;7,"À rechercher",IF(AG151&gt;=75,"P1",IF(AG151&gt;=60,"P2",IF(AG151&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI151" s="31"/>
@@ -11805,7 +11839,7 @@
         <x:f>IF(AF152&gt;=7,SUM(V152:AE152),"")</x:f>
       </x:c>
       <x:c r="AH152" s="33" t="str">
-        <x:f>IF(AF152&lt;7,"À rechercher",IF(AG152&gt;=75,"P147",IF(AG152&gt;=60,"P148",IF(AG152&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF152&lt;7,"À rechercher",IF(AG152&gt;=75,"P1",IF(AG152&gt;=60,"P2",IF(AG152&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI152" s="31"/>
@@ -11876,7 +11910,7 @@
         <x:f>IF(AF153&gt;=7,SUM(V153:AE153),"")</x:f>
       </x:c>
       <x:c r="AH153" s="33" t="str">
-        <x:f>IF(AF153&lt;7,"À rechercher",IF(AG153&gt;=75,"P148",IF(AG153&gt;=60,"P149",IF(AG153&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF153&lt;7,"À rechercher",IF(AG153&gt;=75,"P1",IF(AG153&gt;=60,"P2",IF(AG153&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI153" s="31"/>
@@ -11947,7 +11981,7 @@
         <x:f>IF(AF154&gt;=7,SUM(V154:AE154),"")</x:f>
       </x:c>
       <x:c r="AH154" s="33" t="str">
-        <x:f>IF(AF154&lt;7,"À rechercher",IF(AG154&gt;=75,"P149",IF(AG154&gt;=60,"P150",IF(AG154&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF154&lt;7,"À rechercher",IF(AG154&gt;=75,"P1",IF(AG154&gt;=60,"P2",IF(AG154&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI154" s="31"/>
@@ -12018,7 +12052,7 @@
         <x:f>IF(AF155&gt;=7,SUM(V155:AE155),"")</x:f>
       </x:c>
       <x:c r="AH155" s="33" t="str">
-        <x:f>IF(AF155&lt;7,"À rechercher",IF(AG155&gt;=75,"P150",IF(AG155&gt;=60,"P151",IF(AG155&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF155&lt;7,"À rechercher",IF(AG155&gt;=75,"P1",IF(AG155&gt;=60,"P2",IF(AG155&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI155" s="31"/>
@@ -12089,7 +12123,7 @@
         <x:f>IF(AF156&gt;=7,SUM(V156:AE156),"")</x:f>
       </x:c>
       <x:c r="AH156" s="33" t="str">
-        <x:f>IF(AF156&lt;7,"À rechercher",IF(AG156&gt;=75,"P151",IF(AG156&gt;=60,"P152",IF(AG156&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF156&lt;7,"À rechercher",IF(AG156&gt;=75,"P1",IF(AG156&gt;=60,"P2",IF(AG156&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI156" s="31"/>
@@ -12160,7 +12194,7 @@
         <x:f>IF(AF157&gt;=7,SUM(V157:AE157),"")</x:f>
       </x:c>
       <x:c r="AH157" s="33" t="str">
-        <x:f>IF(AF157&lt;7,"À rechercher",IF(AG157&gt;=75,"P152",IF(AG157&gt;=60,"P153",IF(AG157&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF157&lt;7,"À rechercher",IF(AG157&gt;=75,"P1",IF(AG157&gt;=60,"P2",IF(AG157&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI157" s="31"/>
@@ -12231,7 +12265,7 @@
         <x:f>IF(AF158&gt;=7,SUM(V158:AE158),"")</x:f>
       </x:c>
       <x:c r="AH158" s="33" t="str">
-        <x:f>IF(AF158&lt;7,"À rechercher",IF(AG158&gt;=75,"P153",IF(AG158&gt;=60,"P154",IF(AG158&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF158&lt;7,"À rechercher",IF(AG158&gt;=75,"P1",IF(AG158&gt;=60,"P2",IF(AG158&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI158" s="31"/>
@@ -12302,7 +12336,7 @@
         <x:f>IF(AF159&gt;=7,SUM(V159:AE159),"")</x:f>
       </x:c>
       <x:c r="AH159" s="33" t="str">
-        <x:f>IF(AF159&lt;7,"À rechercher",IF(AG159&gt;=75,"P154",IF(AG159&gt;=60,"P155",IF(AG159&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF159&lt;7,"À rechercher",IF(AG159&gt;=75,"P1",IF(AG159&gt;=60,"P2",IF(AG159&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI159" s="31"/>
@@ -12373,7 +12407,7 @@
         <x:f>IF(AF160&gt;=7,SUM(V160:AE160),"")</x:f>
       </x:c>
       <x:c r="AH160" s="33" t="str">
-        <x:f>IF(AF160&lt;7,"À rechercher",IF(AG160&gt;=75,"P155",IF(AG160&gt;=60,"P156",IF(AG160&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF160&lt;7,"À rechercher",IF(AG160&gt;=75,"P1",IF(AG160&gt;=60,"P2",IF(AG160&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI160" s="31"/>
@@ -12444,7 +12478,7 @@
         <x:f>IF(AF161&gt;=7,SUM(V161:AE161),"")</x:f>
       </x:c>
       <x:c r="AH161" s="33" t="str">
-        <x:f>IF(AF161&lt;7,"À rechercher",IF(AG161&gt;=75,"P156",IF(AG161&gt;=60,"P157",IF(AG161&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF161&lt;7,"À rechercher",IF(AG161&gt;=75,"P1",IF(AG161&gt;=60,"P2",IF(AG161&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI161" s="31"/>
@@ -12515,7 +12549,7 @@
         <x:f>IF(AF162&gt;=7,SUM(V162:AE162),"")</x:f>
       </x:c>
       <x:c r="AH162" s="33" t="str">
-        <x:f>IF(AF162&lt;7,"À rechercher",IF(AG162&gt;=75,"P157",IF(AG162&gt;=60,"P158",IF(AG162&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF162&lt;7,"À rechercher",IF(AG162&gt;=75,"P1",IF(AG162&gt;=60,"P2",IF(AG162&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI162" s="31"/>
@@ -12586,7 +12620,7 @@
         <x:f>IF(AF163&gt;=7,SUM(V163:AE163),"")</x:f>
       </x:c>
       <x:c r="AH163" s="33" t="str">
-        <x:f>IF(AF163&lt;7,"À rechercher",IF(AG163&gt;=75,"P158",IF(AG163&gt;=60,"P159",IF(AG163&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF163&lt;7,"À rechercher",IF(AG163&gt;=75,"P1",IF(AG163&gt;=60,"P2",IF(AG163&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI163" s="31"/>
@@ -12657,7 +12691,7 @@
         <x:f>IF(AF164&gt;=7,SUM(V164:AE164),"")</x:f>
       </x:c>
       <x:c r="AH164" s="33" t="str">
-        <x:f>IF(AF164&lt;7,"À rechercher",IF(AG164&gt;=75,"P159",IF(AG164&gt;=60,"P160",IF(AG164&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF164&lt;7,"À rechercher",IF(AG164&gt;=75,"P1",IF(AG164&gt;=60,"P2",IF(AG164&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI164" s="31"/>
@@ -12728,7 +12762,7 @@
         <x:f>IF(AF165&gt;=7,SUM(V165:AE165),"")</x:f>
       </x:c>
       <x:c r="AH165" s="33" t="str">
-        <x:f>IF(AF165&lt;7,"À rechercher",IF(AG165&gt;=75,"P160",IF(AG165&gt;=60,"P161",IF(AG165&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF165&lt;7,"À rechercher",IF(AG165&gt;=75,"P1",IF(AG165&gt;=60,"P2",IF(AG165&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI165" s="31"/>
@@ -12799,7 +12833,7 @@
         <x:f>IF(AF166&gt;=7,SUM(V166:AE166),"")</x:f>
       </x:c>
       <x:c r="AH166" s="33" t="str">
-        <x:f>IF(AF166&lt;7,"À rechercher",IF(AG166&gt;=75,"P161",IF(AG166&gt;=60,"P162",IF(AG166&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF166&lt;7,"À rechercher",IF(AG166&gt;=75,"P1",IF(AG166&gt;=60,"P2",IF(AG166&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI166" s="31"/>
@@ -12870,7 +12904,7 @@
         <x:f>IF(AF167&gt;=7,SUM(V167:AE167),"")</x:f>
       </x:c>
       <x:c r="AH167" s="33" t="str">
-        <x:f>IF(AF167&lt;7,"À rechercher",IF(AG167&gt;=75,"P162",IF(AG167&gt;=60,"P163",IF(AG167&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF167&lt;7,"À rechercher",IF(AG167&gt;=75,"P1",IF(AG167&gt;=60,"P2",IF(AG167&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI167" s="31"/>
@@ -12941,7 +12975,7 @@
         <x:f>IF(AF168&gt;=7,SUM(V168:AE168),"")</x:f>
       </x:c>
       <x:c r="AH168" s="33" t="str">
-        <x:f>IF(AF168&lt;7,"À rechercher",IF(AG168&gt;=75,"P163",IF(AG168&gt;=60,"P164",IF(AG168&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF168&lt;7,"À rechercher",IF(AG168&gt;=75,"P1",IF(AG168&gt;=60,"P2",IF(AG168&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI168" s="31"/>
@@ -13012,7 +13046,7 @@
         <x:f>IF(AF169&gt;=7,SUM(V169:AE169),"")</x:f>
       </x:c>
       <x:c r="AH169" s="33" t="str">
-        <x:f>IF(AF169&lt;7,"À rechercher",IF(AG169&gt;=75,"P164",IF(AG169&gt;=60,"P165",IF(AG169&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF169&lt;7,"À rechercher",IF(AG169&gt;=75,"P1",IF(AG169&gt;=60,"P2",IF(AG169&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI169" s="31"/>
@@ -13083,7 +13117,7 @@
         <x:f>IF(AF170&gt;=7,SUM(V170:AE170),"")</x:f>
       </x:c>
       <x:c r="AH170" s="33" t="str">
-        <x:f>IF(AF170&lt;7,"À rechercher",IF(AG170&gt;=75,"P165",IF(AG170&gt;=60,"P166",IF(AG170&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF170&lt;7,"À rechercher",IF(AG170&gt;=75,"P1",IF(AG170&gt;=60,"P2",IF(AG170&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI170" s="31"/>
@@ -13154,7 +13188,7 @@
         <x:f>IF(AF171&gt;=7,SUM(V171:AE171),"")</x:f>
       </x:c>
       <x:c r="AH171" s="33" t="str">
-        <x:f>IF(AF171&lt;7,"À rechercher",IF(AG171&gt;=75,"P166",IF(AG171&gt;=60,"P167",IF(AG171&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF171&lt;7,"À rechercher",IF(AG171&gt;=75,"P1",IF(AG171&gt;=60,"P2",IF(AG171&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI171" s="31"/>
@@ -13225,7 +13259,7 @@
         <x:f>IF(AF172&gt;=7,SUM(V172:AE172),"")</x:f>
       </x:c>
       <x:c r="AH172" s="33" t="str">
-        <x:f>IF(AF172&lt;7,"À rechercher",IF(AG172&gt;=75,"P167",IF(AG172&gt;=60,"P168",IF(AG172&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF172&lt;7,"À rechercher",IF(AG172&gt;=75,"P1",IF(AG172&gt;=60,"P2",IF(AG172&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI172" s="31"/>
@@ -13296,7 +13330,7 @@
         <x:f>IF(AF173&gt;=7,SUM(V173:AE173),"")</x:f>
       </x:c>
       <x:c r="AH173" s="33" t="str">
-        <x:f>IF(AF173&lt;7,"À rechercher",IF(AG173&gt;=75,"P168",IF(AG173&gt;=60,"P169",IF(AG173&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF173&lt;7,"À rechercher",IF(AG173&gt;=75,"P1",IF(AG173&gt;=60,"P2",IF(AG173&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI173" s="31"/>
@@ -13367,7 +13401,7 @@
         <x:f>IF(AF174&gt;=7,SUM(V174:AE174),"")</x:f>
       </x:c>
       <x:c r="AH174" s="33" t="str">
-        <x:f>IF(AF174&lt;7,"À rechercher",IF(AG174&gt;=75,"P169",IF(AG174&gt;=60,"P170",IF(AG174&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF174&lt;7,"À rechercher",IF(AG174&gt;=75,"P1",IF(AG174&gt;=60,"P2",IF(AG174&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI174" s="31"/>
@@ -13438,7 +13472,7 @@
         <x:f>IF(AF175&gt;=7,SUM(V175:AE175),"")</x:f>
       </x:c>
       <x:c r="AH175" s="33" t="str">
-        <x:f>IF(AF175&lt;7,"À rechercher",IF(AG175&gt;=75,"P170",IF(AG175&gt;=60,"P171",IF(AG175&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF175&lt;7,"À rechercher",IF(AG175&gt;=75,"P1",IF(AG175&gt;=60,"P2",IF(AG175&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI175" s="31"/>
@@ -13509,7 +13543,7 @@
         <x:f>IF(AF176&gt;=7,SUM(V176:AE176),"")</x:f>
       </x:c>
       <x:c r="AH176" s="33" t="str">
-        <x:f>IF(AF176&lt;7,"À rechercher",IF(AG176&gt;=75,"P171",IF(AG176&gt;=60,"P172",IF(AG176&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF176&lt;7,"À rechercher",IF(AG176&gt;=75,"P1",IF(AG176&gt;=60,"P2",IF(AG176&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI176" s="31"/>
@@ -13580,7 +13614,7 @@
         <x:f>IF(AF177&gt;=7,SUM(V177:AE177),"")</x:f>
       </x:c>
       <x:c r="AH177" s="33" t="str">
-        <x:f>IF(AF177&lt;7,"À rechercher",IF(AG177&gt;=75,"P172",IF(AG177&gt;=60,"P173",IF(AG177&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF177&lt;7,"À rechercher",IF(AG177&gt;=75,"P1",IF(AG177&gt;=60,"P2",IF(AG177&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI177" s="31"/>
@@ -13651,7 +13685,7 @@
         <x:f>IF(AF178&gt;=7,SUM(V178:AE178),"")</x:f>
       </x:c>
       <x:c r="AH178" s="33" t="str">
-        <x:f>IF(AF178&lt;7,"À rechercher",IF(AG178&gt;=75,"P173",IF(AG178&gt;=60,"P174",IF(AG178&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF178&lt;7,"À rechercher",IF(AG178&gt;=75,"P1",IF(AG178&gt;=60,"P2",IF(AG178&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI178" s="31"/>
@@ -13722,7 +13756,7 @@
         <x:f>IF(AF179&gt;=7,SUM(V179:AE179),"")</x:f>
       </x:c>
       <x:c r="AH179" s="33" t="str">
-        <x:f>IF(AF179&lt;7,"À rechercher",IF(AG179&gt;=75,"P174",IF(AG179&gt;=60,"P175",IF(AG179&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF179&lt;7,"À rechercher",IF(AG179&gt;=75,"P1",IF(AG179&gt;=60,"P2",IF(AG179&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI179" s="31"/>
@@ -13793,7 +13827,7 @@
         <x:f>IF(AF180&gt;=7,SUM(V180:AE180),"")</x:f>
       </x:c>
       <x:c r="AH180" s="33" t="str">
-        <x:f>IF(AF180&lt;7,"À rechercher",IF(AG180&gt;=75,"P175",IF(AG180&gt;=60,"P176",IF(AG180&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF180&lt;7,"À rechercher",IF(AG180&gt;=75,"P1",IF(AG180&gt;=60,"P2",IF(AG180&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI180" s="31"/>
@@ -13864,7 +13898,7 @@
         <x:f>IF(AF181&gt;=7,SUM(V181:AE181),"")</x:f>
       </x:c>
       <x:c r="AH181" s="33" t="str">
-        <x:f>IF(AF181&lt;7,"À rechercher",IF(AG181&gt;=75,"P176",IF(AG181&gt;=60,"P177",IF(AG181&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF181&lt;7,"À rechercher",IF(AG181&gt;=75,"P1",IF(AG181&gt;=60,"P2",IF(AG181&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI181" s="31"/>
@@ -13935,7 +13969,7 @@
         <x:f>IF(AF182&gt;=7,SUM(V182:AE182),"")</x:f>
       </x:c>
       <x:c r="AH182" s="33" t="str">
-        <x:f>IF(AF182&lt;7,"À rechercher",IF(AG182&gt;=75,"P177",IF(AG182&gt;=60,"P178",IF(AG182&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF182&lt;7,"À rechercher",IF(AG182&gt;=75,"P1",IF(AG182&gt;=60,"P2",IF(AG182&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI182" s="31"/>
@@ -14006,7 +14040,7 @@
         <x:f>IF(AF183&gt;=7,SUM(V183:AE183),"")</x:f>
       </x:c>
       <x:c r="AH183" s="33" t="str">
-        <x:f>IF(AF183&lt;7,"À rechercher",IF(AG183&gt;=75,"P178",IF(AG183&gt;=60,"P179",IF(AG183&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF183&lt;7,"À rechercher",IF(AG183&gt;=75,"P1",IF(AG183&gt;=60,"P2",IF(AG183&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI183" s="31"/>
@@ -14077,7 +14111,7 @@
         <x:f>IF(AF184&gt;=7,SUM(V184:AE184),"")</x:f>
       </x:c>
       <x:c r="AH184" s="33" t="str">
-        <x:f>IF(AF184&lt;7,"À rechercher",IF(AG184&gt;=75,"P179",IF(AG184&gt;=60,"P180",IF(AG184&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF184&lt;7,"À rechercher",IF(AG184&gt;=75,"P1",IF(AG184&gt;=60,"P2",IF(AG184&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI184" s="31"/>
@@ -14148,7 +14182,7 @@
         <x:f>IF(AF185&gt;=7,SUM(V185:AE185),"")</x:f>
       </x:c>
       <x:c r="AH185" s="33" t="str">
-        <x:f>IF(AF185&lt;7,"À rechercher",IF(AG185&gt;=75,"P180",IF(AG185&gt;=60,"P181",IF(AG185&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF185&lt;7,"À rechercher",IF(AG185&gt;=75,"P1",IF(AG185&gt;=60,"P2",IF(AG185&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI185" s="31"/>
@@ -14219,7 +14253,7 @@
         <x:f>IF(AF186&gt;=7,SUM(V186:AE186),"")</x:f>
       </x:c>
       <x:c r="AH186" s="33" t="str">
-        <x:f>IF(AF186&lt;7,"À rechercher",IF(AG186&gt;=75,"P181",IF(AG186&gt;=60,"P182",IF(AG186&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF186&lt;7,"À rechercher",IF(AG186&gt;=75,"P1",IF(AG186&gt;=60,"P2",IF(AG186&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI186" s="31"/>
@@ -14290,7 +14324,7 @@
         <x:f>IF(AF187&gt;=7,SUM(V187:AE187),"")</x:f>
       </x:c>
       <x:c r="AH187" s="33" t="str">
-        <x:f>IF(AF187&lt;7,"À rechercher",IF(AG187&gt;=75,"P182",IF(AG187&gt;=60,"P183",IF(AG187&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF187&lt;7,"À rechercher",IF(AG187&gt;=75,"P1",IF(AG187&gt;=60,"P2",IF(AG187&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI187" s="31"/>
@@ -14361,7 +14395,7 @@
         <x:f>IF(AF188&gt;=7,SUM(V188:AE188),"")</x:f>
       </x:c>
       <x:c r="AH188" s="33" t="str">
-        <x:f>IF(AF188&lt;7,"À rechercher",IF(AG188&gt;=75,"P183",IF(AG188&gt;=60,"P184",IF(AG188&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF188&lt;7,"À rechercher",IF(AG188&gt;=75,"P1",IF(AG188&gt;=60,"P2",IF(AG188&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI188" s="31"/>
@@ -14432,7 +14466,7 @@
         <x:f>IF(AF189&gt;=7,SUM(V189:AE189),"")</x:f>
       </x:c>
       <x:c r="AH189" s="33" t="str">
-        <x:f>IF(AF189&lt;7,"À rechercher",IF(AG189&gt;=75,"P184",IF(AG189&gt;=60,"P185",IF(AG189&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF189&lt;7,"À rechercher",IF(AG189&gt;=75,"P1",IF(AG189&gt;=60,"P2",IF(AG189&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI189" s="31"/>
@@ -14503,7 +14537,7 @@
         <x:f>IF(AF190&gt;=7,SUM(V190:AE190),"")</x:f>
       </x:c>
       <x:c r="AH190" s="33" t="str">
-        <x:f>IF(AF190&lt;7,"À rechercher",IF(AG190&gt;=75,"P185",IF(AG190&gt;=60,"P186",IF(AG190&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF190&lt;7,"À rechercher",IF(AG190&gt;=75,"P1",IF(AG190&gt;=60,"P2",IF(AG190&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI190" s="31"/>
@@ -14574,7 +14608,7 @@
         <x:f>IF(AF191&gt;=7,SUM(V191:AE191),"")</x:f>
       </x:c>
       <x:c r="AH191" s="33" t="str">
-        <x:f>IF(AF191&lt;7,"À rechercher",IF(AG191&gt;=75,"P186",IF(AG191&gt;=60,"P187",IF(AG191&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF191&lt;7,"À rechercher",IF(AG191&gt;=75,"P1",IF(AG191&gt;=60,"P2",IF(AG191&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI191" s="31"/>
@@ -14645,7 +14679,7 @@
         <x:f>IF(AF192&gt;=7,SUM(V192:AE192),"")</x:f>
       </x:c>
       <x:c r="AH192" s="33" t="str">
-        <x:f>IF(AF192&lt;7,"À rechercher",IF(AG192&gt;=75,"P187",IF(AG192&gt;=60,"P188",IF(AG192&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF192&lt;7,"À rechercher",IF(AG192&gt;=75,"P1",IF(AG192&gt;=60,"P2",IF(AG192&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI192" s="31"/>
@@ -14716,7 +14750,7 @@
         <x:f>IF(AF193&gt;=7,SUM(V193:AE193),"")</x:f>
       </x:c>
       <x:c r="AH193" s="33" t="str">
-        <x:f>IF(AF193&lt;7,"À rechercher",IF(AG193&gt;=75,"P188",IF(AG193&gt;=60,"P189",IF(AG193&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF193&lt;7,"À rechercher",IF(AG193&gt;=75,"P1",IF(AG193&gt;=60,"P2",IF(AG193&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI193" s="31"/>
@@ -14787,7 +14821,7 @@
         <x:f>IF(AF194&gt;=7,SUM(V194:AE194),"")</x:f>
       </x:c>
       <x:c r="AH194" s="33" t="str">
-        <x:f>IF(AF194&lt;7,"À rechercher",IF(AG194&gt;=75,"P189",IF(AG194&gt;=60,"P190",IF(AG194&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF194&lt;7,"À rechercher",IF(AG194&gt;=75,"P1",IF(AG194&gt;=60,"P2",IF(AG194&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI194" s="31"/>
@@ -14858,7 +14892,7 @@
         <x:f>IF(AF195&gt;=7,SUM(V195:AE195),"")</x:f>
       </x:c>
       <x:c r="AH195" s="33" t="str">
-        <x:f>IF(AF195&lt;7,"À rechercher",IF(AG195&gt;=75,"P190",IF(AG195&gt;=60,"P191",IF(AG195&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF195&lt;7,"À rechercher",IF(AG195&gt;=75,"P1",IF(AG195&gt;=60,"P2",IF(AG195&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI195" s="31"/>
@@ -14929,7 +14963,7 @@
         <x:f>IF(AF196&gt;=7,SUM(V196:AE196),"")</x:f>
       </x:c>
       <x:c r="AH196" s="33" t="str">
-        <x:f>IF(AF196&lt;7,"À rechercher",IF(AG196&gt;=75,"P191",IF(AG196&gt;=60,"P192",IF(AG196&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF196&lt;7,"À rechercher",IF(AG196&gt;=75,"P1",IF(AG196&gt;=60,"P2",IF(AG196&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI196" s="31"/>
@@ -15000,7 +15034,7 @@
         <x:f>IF(AF197&gt;=7,SUM(V197:AE197),"")</x:f>
       </x:c>
       <x:c r="AH197" s="33" t="str">
-        <x:f>IF(AF197&lt;7,"À rechercher",IF(AG197&gt;=75,"P192",IF(AG197&gt;=60,"P193",IF(AG197&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF197&lt;7,"À rechercher",IF(AG197&gt;=75,"P1",IF(AG197&gt;=60,"P2",IF(AG197&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI197" s="31"/>
@@ -15071,7 +15105,7 @@
         <x:f>IF(AF198&gt;=7,SUM(V198:AE198),"")</x:f>
       </x:c>
       <x:c r="AH198" s="33" t="str">
-        <x:f>IF(AF198&lt;7,"À rechercher",IF(AG198&gt;=75,"P193",IF(AG198&gt;=60,"P194",IF(AG198&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF198&lt;7,"À rechercher",IF(AG198&gt;=75,"P1",IF(AG198&gt;=60,"P2",IF(AG198&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI198" s="31"/>
@@ -15142,7 +15176,7 @@
         <x:f>IF(AF199&gt;=7,SUM(V199:AE199),"")</x:f>
       </x:c>
       <x:c r="AH199" s="33" t="str">
-        <x:f>IF(AF199&lt;7,"À rechercher",IF(AG199&gt;=75,"P194",IF(AG199&gt;=60,"P195",IF(AG199&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF199&lt;7,"À rechercher",IF(AG199&gt;=75,"P1",IF(AG199&gt;=60,"P2",IF(AG199&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI199" s="31"/>
@@ -15213,7 +15247,7 @@
         <x:f>IF(AF200&gt;=7,SUM(V200:AE200),"")</x:f>
       </x:c>
       <x:c r="AH200" s="33" t="str">
-        <x:f>IF(AF200&lt;7,"À rechercher",IF(AG200&gt;=75,"P195",IF(AG200&gt;=60,"P196",IF(AG200&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF200&lt;7,"À rechercher",IF(AG200&gt;=75,"P1",IF(AG200&gt;=60,"P2",IF(AG200&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI200" s="31"/>
@@ -15284,7 +15318,7 @@
         <x:f>IF(AF201&gt;=7,SUM(V201:AE201),"")</x:f>
       </x:c>
       <x:c r="AH201" s="33" t="str">
-        <x:f>IF(AF201&lt;7,"À rechercher",IF(AG201&gt;=75,"P196",IF(AG201&gt;=60,"P197",IF(AG201&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF201&lt;7,"À rechercher",IF(AG201&gt;=75,"P1",IF(AG201&gt;=60,"P2",IF(AG201&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI201" s="31"/>
@@ -15355,7 +15389,7 @@
         <x:f>IF(AF202&gt;=7,SUM(V202:AE202),"")</x:f>
       </x:c>
       <x:c r="AH202" s="33" t="str">
-        <x:f>IF(AF202&lt;7,"À rechercher",IF(AG202&gt;=75,"P197",IF(AG202&gt;=60,"P198",IF(AG202&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF202&lt;7,"À rechercher",IF(AG202&gt;=75,"P1",IF(AG202&gt;=60,"P2",IF(AG202&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI202" s="31"/>
@@ -15426,7 +15460,7 @@
         <x:f>IF(AF203&gt;=7,SUM(V203:AE203),"")</x:f>
       </x:c>
       <x:c r="AH203" s="33" t="str">
-        <x:f>IF(AF203&lt;7,"À rechercher",IF(AG203&gt;=75,"P198",IF(AG203&gt;=60,"P199",IF(AG203&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF203&lt;7,"À rechercher",IF(AG203&gt;=75,"P1",IF(AG203&gt;=60,"P2",IF(AG203&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI203" s="31"/>
@@ -15497,7 +15531,7 @@
         <x:f>IF(AF204&gt;=7,SUM(V204:AE204),"")</x:f>
       </x:c>
       <x:c r="AH204" s="33" t="str">
-        <x:f>IF(AF204&lt;7,"À rechercher",IF(AG204&gt;=75,"P199",IF(AG204&gt;=60,"P200",IF(AG204&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF204&lt;7,"À rechercher",IF(AG204&gt;=75,"P1",IF(AG204&gt;=60,"P2",IF(AG204&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI204" s="31"/>
@@ -15568,7 +15602,7 @@
         <x:f>IF(AF205&gt;=7,SUM(V205:AE205),"")</x:f>
       </x:c>
       <x:c r="AH205" s="33" t="str">
-        <x:f>IF(AF205&lt;7,"À rechercher",IF(AG205&gt;=75,"P200",IF(AG205&gt;=60,"P201",IF(AG205&gt;=45,"À enrichir","Faible priorité"))))</x:f>
+        <x:f>IF(AF205&lt;7,"À rechercher",IF(AG205&gt;=75,"P1",IF(AG205&gt;=60,"P2",IF(AG205&gt;=45,"P3","Faible priorité"))))</x:f>
         <x:v>À rechercher</x:v>
       </x:c>
       <x:c r="AI205" s="31"/>
@@ -15611,7 +15645,7 @@
   <x:conditionalFormatting sqref="C6:C205">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="P1"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="9">
+  <x:dataValidations count="11">
     <x:dataValidation type="list" sqref="B6:B205">
       <x:formula1>'LISTES'!$A$6:$A$8</x:formula1>
     </x:dataValidation>
@@ -15639,10 +15673,16 @@
     <x:dataValidation type="list" sqref="BE6:BE205">
       <x:formula1>'LISTES'!$J$6:$J$7</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="C6:C205">
+      <x:formula1>'LISTES'!$B$6:$B$10</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AT6:AT205">
+      <x:formula1>'LISTES'!$O$6:$O$6</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abade65deca4b0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ccbc1c6c6b44f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23249,7 +23289,7 @@
   <x:conditionalFormatting sqref="M6:M505">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Oui"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="5">
+  <x:dataValidations count="6">
     <x:dataValidation type="list" sqref="C6:C505">
       <x:formula1>'LISTES'!$A$6:$A$8</x:formula1>
     </x:dataValidation>
@@ -23265,10 +23305,13 @@
     <x:dataValidation type="list" sqref="M6:M505">
       <x:formula1>'LISTES'!$J$6:$J$7</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="L6:L505">
+      <x:formula1>'LISTES'!$O$6:$O$6</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a491debc8b3424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d56ac735bbb41a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23346,7 +23389,7 @@
         <x:v>STATUT</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>TRAITEE_PAR</x:v>
+        <x:v>ENTREPRISE_SI_UTILE</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -25368,7 +25411,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c7e921824ad42d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2308fbbe8ac64ff4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25712,6 +25755,7 @@
     <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -25793,6 +25837,9 @@
       <x:c r="N5" s="17" t="str">
         <x:v>STATUT_OPPOSITION</x:v>
       </x:c>
+      <x:c r="O5" s="82" t="str">
+        <x:v>RESPONSABLES</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="str">
@@ -25835,7 +25882,10 @@
         <x:v>E-mail professionnel</x:v>
       </x:c>
       <x:c r="N6" s="20" t="str">
-        <x:v>Ne plus contacter</x:v>
+        <x:v>NE PLUS CONTACTER</x:v>
+      </x:c>
+      <x:c r="O6" s="83" t="str">
+        <x:v>Julien GREGUREC</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -25885,7 +25935,7 @@
         <x:v>Lot 3</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>À enrichir</x:v>
+        <x:v>P3</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
         <x:v>À contacter</x:v>

</xml_diff>